<commit_message>
Complete US-011 realtime single-note playback
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rdc708d6d2b944c02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rac577e90d0354fdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R63f590b772cc4d17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rc70ab57d807b40db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R2433202b8d784554"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R58295e8514cd4531"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R6bc14e3214644a47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R58712bea3e604481"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1171,7 +1171,7 @@
         <x:v>Play Single Note</x:v>
       </x:c>
       <x:c r="E15" s="16" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F15" s="16" t="str">
         <x:v>Must</x:v>
@@ -1186,19 +1186,19 @@
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="J15" s="16" t="str">
-        <x:v>play --note C3 maakt hoorbaar geluid.</x:v>
+        <x:v>play --note C3 maakt hoorbaar geluid en kan --audio-device gebruiken.</x:v>
       </x:c>
       <x:c r="K15" s="16" t="str">
-        <x:v>Audio output adapter test faalt.</x:v>
+        <x:v>Audio output adapter en CLI parsing tests falen.</x:v>
       </x:c>
       <x:c r="L15" s="16" t="str">
-        <x:v>sounddevice adapter en CLI play command.</x:v>
+        <x:v>sounddevice adapter, audio list-devices, --audio-device en Scarlett testdocs.</x:v>
       </x:c>
       <x:c r="M15" s="16" t="str">
         <x:v>US-007</x:v>
       </x:c>
       <x:c r="N15" s="18" t="str">
-        <x:v>Adapter aanwezig; hoorbare output nog niet handmatig geverifieerd.</x:v>
+        <x:v>Klanttest geslaagd: hoorbaar geluid via Scarlett 8i6 USB.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9020d42033304cb0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red6b7188f6064918"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1925,19 +1925,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J11" s="40" t="str">
-        <x:v>CLI scant MIDI devices en kiest device via CLI of YAML default.</x:v>
+        <x:v>CLI scant MIDI devices veilig en kiest device via CLI of YAML default.</x:v>
       </x:c>
       <x:c r="K11" s="40" t="str">
         <x:v>Device discovery en config precedence tests falen.</x:v>
       </x:c>
       <x:c r="L11" s="40" t="str">
-        <x:v>MidiDeviceScanner, CLI list-devices en config default.</x:v>
+        <x:v>MidiDeviceScanner met veilige macOS default en optionele --unsafe-rtmidi-scan.</x:v>
       </x:c>
       <x:c r="M11" s="40" t="str">
         <x:v>US-019, US-020, US-022</x:v>
       </x:c>
       <x:c r="N11" s="42" t="str">
-        <x:v>Skeleton toegevoegd; optionele mido/backend nog nodig voor echte devices.</x:v>
+        <x:v>RtMidi/CoreMIDI crashrapporten voorkomen door native scan standaard uit te schakelen.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a7fcf2497674055"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R907b900504b84e7d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2014,11 +2014,11 @@
       </x:c>
       <x:c r="E4" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,D4)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F4" s="44" t="n">
         <x:f>SUMIF('Sprint 1 Board'!E5:E22,D4,'Sprint 1 Board'!H5:H22)</x:f>
-        <x:v>8</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2074,11 +2074,11 @@
       </x:c>
       <x:c r="E7" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,D7)</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F7" s="44" t="n">
         <x:f>SUMIF('Sprint 1 Board'!E5:E22,D7,'Sprint 1 Board'!H5:H22)</x:f>
-        <x:v>33</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="8">

</xml_diff>

<commit_message>
Complete US-012 testsequence playback
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R2433202b8d784554"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R58295e8514cd4531"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R6bc14e3214644a47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R58712bea3e604481"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rb512885428a54dd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R2916bf9ee41d4a7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R77bd0c7a57c845d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R7dd64acc23b545d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1215,7 +1215,7 @@
         <x:v>Play Testsequence</x:v>
       </x:c>
       <x:c r="E16" s="16" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F16" s="16" t="str">
         <x:v>Must</x:v>
@@ -1230,19 +1230,19 @@
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="J16" s="16" t="str">
-        <x:v>play --testsequence ACGD speelt vier noten.</x:v>
+        <x:v>play --testsequence ACGD speelt vier noten en ondersteunt --audio-device.</x:v>
       </x:c>
       <x:c r="K16" s="16" t="str">
         <x:v>Sequence playback test faalt.</x:v>
       </x:c>
       <x:c r="L16" s="16" t="str">
-        <x:v>Playback engine voor NoteSequence.</x:v>
+        <x:v>Playback engine voor NoteSequence plus CLI verbose eventdiagnose.</x:v>
       </x:c>
       <x:c r="M16" s="16" t="str">
         <x:v>US-005, US-011</x:v>
       </x:c>
       <x:c r="N16" s="18" t="str">
-        <x:v>Dumb user testmode.</x:v>
+        <x:v>Klanttest geslaagd: ACGD sequence hoorbaar via Scarlett 8i6 USB.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red6b7188f6064918"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89fa60ceabaa442f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R907b900504b84e7d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9986c5cb10a24fef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2014,11 +2014,11 @@
       </x:c>
       <x:c r="E4" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,D4)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F4" s="44" t="n">
         <x:f>SUMIF('Sprint 1 Board'!E5:E22,D4,'Sprint 1 Board'!H5:H22)</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -2074,11 +2074,11 @@
       </x:c>
       <x:c r="E7" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,D7)</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F7" s="44" t="n">
         <x:f>SUMIF('Sprint 1 Board'!E5:E22,D7,'Sprint 1 Board'!H5:H22)</x:f>
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="8">

</xml_diff>

<commit_message>
Complete US-013 channel selection
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rb512885428a54dd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R2916bf9ee41d4a7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R77bd0c7a57c845d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R7dd64acc23b545d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R4f343a8a5a7e4ee9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R592af428803f485f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rab06b7ab33be416f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rec1d806cba1b48a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1259,7 +1259,7 @@
         <x:v>Channel Selection</x:v>
       </x:c>
       <x:c r="E17" s="16" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F17" s="16" t="str">
         <x:v>Must</x:v>
@@ -1274,19 +1274,19 @@
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="J17" s="16" t="str">
-        <x:v>stereo/left/right kanaalrouting werkt.</x:v>
+        <x:v>stereo/left/right kanaalrouting werkt met traceerbare code-docstrings.</x:v>
       </x:c>
       <x:c r="K17" s="16" t="str">
-        <x:v>Kanaalrouting tests falen.</x:v>
+        <x:v>Kanaalrouting en traceability tests falen.</x:v>
       </x:c>
       <x:c r="L17" s="16" t="str">
-        <x:v>ChannelRouter class en CLI option.</x:v>
+        <x:v>ChannelRouter, SynthEngine en CLI tests voor stereo/left/right plus code traceability.</x:v>
       </x:c>
       <x:c r="M17" s="16" t="str">
         <x:v>US-010, US-011</x:v>
       </x:c>
       <x:c r="N17" s="18" t="str">
-        <x:v>ChannelRouter en test aangemaakt.</x:v>
+        <x:v>Klanttest geslaagd: stereo, left en right hoorbaar via Scarlett 8i6 USB.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89fa60ceabaa442f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8400e7820ec24e82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9986c5cb10a24fef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3257b8ab4644c2a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2054,11 +2054,11 @@
       </x:c>
       <x:c r="E6" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,D6)</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F6" s="44" t="n">
         <x:f>SUMIF('Sprint 1 Board'!E5:E22,D6,'Sprint 1 Board'!H5:H22)</x:f>
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2074,11 +2074,11 @@
       </x:c>
       <x:c r="E7" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,D7)</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F7" s="44" t="n">
         <x:f>SUMIF('Sprint 1 Board'!E5:E22,D7,'Sprint 1 Board'!H5:H22)</x:f>
-        <x:v>41</x:v>
+        <x:v>44</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2087,7 +2087,7 @@
       </x:c>
       <x:c r="B8" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,"In Review")</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D8" s="44" t="str">
         <x:v>Blocked</x:v>

</xml_diff>

<commit_message>
Complete US-006 note event model
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R7809fd1b32db463b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R2984435eaf6b4bd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R6455eab599354640"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R3ecab413cbf34678"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R3be6931d8ed14829"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R08cf181cb51b409f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R90d92e42ed514387"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Raba0ee04f6ee4158"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -951,7 +951,7 @@
         <x:v>NoteEvent En NoteSequence Model</x:v>
       </x:c>
       <x:c r="E10" s="16" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F10" s="16" t="str">
         <x:v>Must</x:v>
@@ -966,19 +966,19 @@
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="J10" s="16" t="str">
-        <x:v>Intern eventmodel ondersteunt note, duration, velocity en timing.</x:v>
+        <x:v>Intern eventmodel ondersteunt note, duration, velocity, timing en traceerbare code-docstrings.</x:v>
       </x:c>
       <x:c r="K10" s="16" t="str">
-        <x:v>Modelvalidatie tests falen.</x:v>
+        <x:v>Modelvalidatie en traceability tests falen.</x:v>
       </x:c>
       <x:c r="L10" s="16" t="str">
-        <x:v>Class based event/sequence model.</x:v>
+        <x:v>NoteEvent validatie, NoteSequence tuple-normalisatie en code traceability.</x:v>
       </x:c>
       <x:c r="M10" s="16" t="str">
         <x:v>US-004</x:v>
       </x:c>
       <x:c r="N10" s="18" t="str">
-        <x:v>Dataclasses toegevoegd als basis voor MIDI mapping.</x:v>
+        <x:v>pytest groen: duration, velocity, timing, volgorde en traceability afgedekt.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbdc76ec3d704ef1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R855366e78f9a48c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0365c20e7d734d90"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R234a6bc96e2546d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2054,11 +2054,11 @@
       </x:c>
       <x:c r="E6" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,D6)</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F6" s="44" t="n">
         <x:f>SUMIF('Sprint 1 Board'!E5:E22,D6,'Sprint 1 Board'!H5:H22)</x:f>
-        <x:v>9</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2074,11 +2074,11 @@
       </x:c>
       <x:c r="E7" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,D7)</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="F7" s="44" t="n">
         <x:f>SUMIF('Sprint 1 Board'!E5:E22,D7,'Sprint 1 Board'!H5:H22)</x:f>
-        <x:v>46</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2087,7 +2087,7 @@
       </x:c>
       <x:c r="B8" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,"In Review")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D8" s="44" t="str">
         <x:v>Blocked</x:v>

</xml_diff>

<commit_message>
Complete US-009 square oscillator
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R3be6931d8ed14829"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R08cf181cb51b409f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R90d92e42ed514387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Raba0ee04f6ee4158"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R21f41b6bce0d4990"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R2ea764c91ed84420"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R02eb941e747f4a97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R8b58ff7f59384a14"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1083,7 +1083,7 @@
         <x:v>Square Oscillator</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F13" s="16" t="str">
         <x:v>Should</x:v>
@@ -1098,19 +1098,19 @@
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="J13" s="16" t="str">
-        <x:v>Square samples hebben juiste lengte en amplitude.</x:v>
+        <x:v>Square samples hebben juiste lengte, amplitude en discrete niveaus met traceerbare code-docstrings.</x:v>
       </x:c>
       <x:c r="K13" s="16" t="str">
-        <x:v>Square oscillator tests falen.</x:v>
+        <x:v>Square oscillator en traceability tests falen.</x:v>
       </x:c>
       <x:c r="L13" s="16" t="str">
-        <x:v>SquareOscillator class.</x:v>
+        <x:v>Oscillator ondersteunt square met discrete -amplitude/+amplitude output.</x:v>
       </x:c>
       <x:c r="M13" s="16" t="str">
         <x:v>US-007</x:v>
       </x:c>
       <x:c r="N13" s="18" t="str">
-        <x:v>Waveform enum en oscillator ondersteunen square.</x:v>
+        <x:v>pytest groen: square count, amplitude, levels en traceability afgedekt.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R855366e78f9a48c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d50a22106a1465b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R234a6bc96e2546d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc04be4abdcfc4b8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2054,11 +2054,11 @@
       </x:c>
       <x:c r="E6" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,D6)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F6" s="44" t="n">
         <x:f>SUMIF('Sprint 1 Board'!E5:E22,D6,'Sprint 1 Board'!H5:H22)</x:f>
-        <x:v>6</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2074,11 +2074,11 @@
       </x:c>
       <x:c r="E7" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,D7)</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F7" s="44" t="n">
         <x:f>SUMIF('Sprint 1 Board'!E5:E22,D7,'Sprint 1 Board'!H5:H22)</x:f>
-        <x:v>49</x:v>
+        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2087,7 +2087,7 @@
       </x:c>
       <x:c r="B8" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,"In Review")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="44" t="str">
         <x:v>Blocked</x:v>

</xml_diff>

<commit_message>
Complete US-008 saw oscillator
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R21f41b6bce0d4990"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R2ea764c91ed84420"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R02eb941e747f4a97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R8b58ff7f59384a14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R4587a2c575db4677"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R252f3be914a044d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R9f603350c6ee41f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rbed74902efe84a46"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1039,7 +1039,7 @@
         <x:v>Saw Oscillator</x:v>
       </x:c>
       <x:c r="E12" s="16" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F12" s="16" t="str">
         <x:v>Should</x:v>
@@ -1054,19 +1054,19 @@
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="J12" s="16" t="str">
-        <x:v>Saw samples hebben juiste lengte en amplitude.</x:v>
+        <x:v>Saw samples hebben juiste lengte, amplitude en ramp-niveaus met traceerbare code-docstrings.</x:v>
       </x:c>
       <x:c r="K12" s="16" t="str">
-        <x:v>Saw oscillator tests falen.</x:v>
+        <x:v>Saw oscillator en traceability tests falen.</x:v>
       </x:c>
       <x:c r="L12" s="16" t="str">
-        <x:v>SawOscillator class.</x:v>
+        <x:v>Oscillator ondersteunt saw met meerdere ramp-niveaus binnen amplitude.</x:v>
       </x:c>
       <x:c r="M12" s="16" t="str">
         <x:v>US-007</x:v>
       </x:c>
       <x:c r="N12" s="18" t="str">
-        <x:v>Waveform enum en oscillator ondersteunen saw.</x:v>
+        <x:v>pytest groen: saw count, amplitude, ramp levels en traceability afgedekt.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d50a22106a1465b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cf99e040543453b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc04be4abdcfc4b8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6b5003d328a4ea5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2054,11 +2054,11 @@
       </x:c>
       <x:c r="E6" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,D6)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="44" t="n">
         <x:f>SUMIF('Sprint 1 Board'!E5:E22,D6,'Sprint 1 Board'!H5:H22)</x:f>
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2074,11 +2074,11 @@
       </x:c>
       <x:c r="E7" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,D7)</x:f>
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="F7" s="44" t="n">
         <x:f>SUMIF('Sprint 1 Board'!E5:E22,D7,'Sprint 1 Board'!H5:H22)</x:f>
-        <x:v>52</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2087,7 +2087,7 @@
       </x:c>
       <x:c r="B8" s="44" t="n">
         <x:f>COUNTIF('Sprint 1 Board'!E5:E22,"In Review")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="44" t="str">
         <x:v>Blocked</x:v>

</xml_diff>

<commit_message>
Complete US-019 midi learning path
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R4587a2c575db4677"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R252f3be914a044d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R9f603350c6ee41f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rbed74902efe84a46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Re02755f5d2c64c23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R80b7b70c03e74f2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R27944b6d08914175"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rbb6665a40d9d44ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cf99e040543453b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5084831e8844cbb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1646,7 +1646,7 @@
         <x:v>MIDI Leerpad En Terminologie</x:v>
       </x:c>
       <x:c r="E5" s="36" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F5" s="36" t="str">
         <x:v>Must</x:v>
@@ -1661,19 +1661,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J5" s="36" t="str">
-        <x:v>Klant begrijpt note on/off, channel, velocity, clock en pitch bend.</x:v>
+        <x:v>Klant begrijpt note on/off, note number, channel, velocity, MIDI clock en pitch bend.</x:v>
       </x:c>
       <x:c r="K5" s="36" t="str">
         <x:v>Docs ontbreken voor MIDI basisbegrippen.</x:v>
       </x:c>
       <x:c r="L5" s="36" t="str">
-        <x:v>MIDI concept guide en glossary.</x:v>
+        <x:v>MIDI concept guide en glossary met NoteEvent mapping.</x:v>
       </x:c>
       <x:c r="M5" s="36" t="str">
         <x:v>US-006</x:v>
       </x:c>
       <x:c r="N5" s="38" t="str">
-        <x:v>Eerst uitleg voordat hardware-integratie start.</x:v>
+        <x:v>docs/midi_learning_path_v0.1.0.md en pytest docs-check groen.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6b5003d328a4ea5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e86ede1be3848d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete US-020 virtual midi input
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Re02755f5d2c64c23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R80b7b70c03e74f2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R27944b6d08914175"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rbb6665a40d9d44ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rea9a5f32b2b34d9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R93c7cd6c4fa04426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R8da2204b6c874b3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rc8804752fef54e86"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5084831e8844cbb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a800bdf62894779"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1690,7 +1690,7 @@
         <x:v>Virtual MIDI Input Voor DAW</x:v>
       </x:c>
       <x:c r="E6" s="36" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F6" s="36" t="str">
         <x:v>Must</x:v>
@@ -1705,19 +1705,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J6" s="36" t="str">
-        <x:v>Logic Pro 12.3 of andere DAW kan note events naar de synth sturen.</x:v>
+        <x:v>Logic Pro 12.3 of andere DAW heeft veilige virtual MIDI input voorbereiding en note-event mapping.</x:v>
       </x:c>
       <x:c r="K6" s="36" t="str">
-        <x:v>Virtual MIDI route test faalt.</x:v>
+        <x:v>Virtual MIDI adapter, CLI diagnose en traceability tests falen.</x:v>
       </x:c>
       <x:c r="L6" s="36" t="str">
-        <x:v>Virtual MIDI input adapter en event bridge.</x:v>
+        <x:v>VirtualMidiInputAdapter, MidiMessage en midi diagnose-virtual-input.</x:v>
       </x:c>
       <x:c r="M6" s="36" t="str">
         <x:v>US-006, US-019</x:v>
       </x:c>
       <x:c r="N6" s="38" t="str">
-        <x:v>Software route naast latere pluginroute.</x:v>
+        <x:v>pytest groen: note on/off mapping, velocity zero note-off, CLI diagnose en traceability.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e86ede1be3848d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra98c82e1ceeb49a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Prepare US-021 logic midi workflow
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rea9a5f32b2b34d9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R93c7cd6c4fa04426"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R8da2204b6c874b3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rc8804752fef54e86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R04f89cf5601e4724"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R10805ed2cc764fe0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rce815f7073aa46ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R4a8705882a3c4e96"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a800bdf62894779"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17cd948a8de14e8c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1734,7 +1734,7 @@
         <x:v>External MIDI Workflow In Logic</x:v>
       </x:c>
       <x:c r="E7" s="36" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="F7" s="36" t="str">
         <x:v>Should</x:v>
@@ -1749,19 +1749,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J7" s="36" t="str">
-        <x:v>External MIDI workflow in Logic is reproduceerbaar beschreven.</x:v>
+        <x:v>External MIDI workflow in Logic is reproduceerbaar beschreven en wacht op klanttest.</x:v>
       </x:c>
       <x:c r="K7" s="36" t="str">
         <x:v>Logic external MIDI setup test faalt of ontbreekt.</x:v>
       </x:c>
       <x:c r="L7" s="36" t="str">
-        <x:v>Setup guide en handmatige DAW test.</x:v>
+        <x:v>Logic/IAC workflowdoc en handmatige testtemplate.</x:v>
       </x:c>
       <x:c r="M7" s="36" t="str">
         <x:v>US-020</x:v>
       </x:c>
       <x:c r="N7" s="38" t="str">
-        <x:v>Logic Pro 12.3 is primaire DAW, maar ontwerp blijft DAW-breed.</x:v>
+        <x:v>docs/logic_external_midi_workflow_v0.1.0.md; wacht op Logic Pro 12.3 testresultaat.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra98c82e1ceeb49a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb885fcab18974b45"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete US-021 logic midi workflow
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R04f89cf5601e4724"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R10805ed2cc764fe0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rce815f7073aa46ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R4a8705882a3c4e96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Re80013c91b0c4c82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R609be9da7f984dec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R5c8fc95c17f0406d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Radb730f84af24206"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17cd948a8de14e8c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb5bfc470c6f428e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1734,7 +1734,7 @@
         <x:v>External MIDI Workflow In Logic</x:v>
       </x:c>
       <x:c r="E7" s="36" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F7" s="36" t="str">
         <x:v>Should</x:v>
@@ -1749,19 +1749,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J7" s="36" t="str">
-        <x:v>External MIDI workflow in Logic is reproduceerbaar beschreven en wacht op klanttest.</x:v>
+        <x:v>External MIDI workflow in Logic is reproduceerbaar beschreven en klanttest is vastgelegd.</x:v>
       </x:c>
       <x:c r="K7" s="36" t="str">
         <x:v>Logic external MIDI setup test faalt of ontbreekt.</x:v>
       </x:c>
       <x:c r="L7" s="36" t="str">
-        <x:v>Logic/IAC workflowdoc en handmatige testtemplate.</x:v>
+        <x:v>Logic/IAC workflowdoc en handmatige testresultaatregistratie.</x:v>
       </x:c>
       <x:c r="M7" s="36" t="str">
         <x:v>US-020</x:v>
       </x:c>
       <x:c r="N7" s="38" t="str">
-        <x:v>docs/logic_external_midi_workflow_v0.1.0.md; wacht op Logic Pro 12.3 testresultaat.</x:v>
+        <x:v>Klanttest geslaagd: IAC route zichtbaar, Python diagnose OK, geen geluid verwacht in US-021.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb885fcab18974b45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85e8499c63484c86"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Prepare US-022 generic usb midi input
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Re80013c91b0c4c82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R609be9da7f984dec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R5c8fc95c17f0406d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Radb730f84af24206"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rb2c45696a1be4a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R21f0849afc174914"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Re7011d3f7fd34734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rcf202a436607413b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb5bfc470c6f428e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b8a862be2d54ef1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1572,7 +1572,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="28" t="str">
-        <x:v>Scope mutation: Logic Pro 12.3, other DAWs, USB MIDI, external MIDI, RaspiMidiHub, physical MIDI hub, MiniFreak, Arturia KeyLab Mk3</x:v>
+        <x:v>Scope mutation: Logic Pro 12.3, other DAWs, generic USB MIDI, external MIDI, RaspiMidiHub, physical MIDI hub, MiniFreak, Arturia KeyLab Mk3, Fishman TriplePlay, M-Vave</x:v>
       </x:c>
       <x:c r="B2" s="28"/>
       <x:c r="C2" s="28"/>
@@ -1778,7 +1778,7 @@
         <x:v>USB MIDI Hardware Input</x:v>
       </x:c>
       <x:c r="E8" s="36" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="F8" s="36" t="str">
         <x:v>Must</x:v>
@@ -1793,19 +1793,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J8" s="36" t="str">
-        <x:v>Arturia KeyLab Mk3 kan note on/off en velocity aanleveren.</x:v>
+        <x:v>Generieke USB MIDI inputdiagnose werkt voor KeyLab, Fishman TriplePlay, M-Vave en andere inputdevices.</x:v>
       </x:c>
       <x:c r="K8" s="36" t="str">
-        <x:v>USB MIDI device detectie test faalt.</x:v>
+        <x:v>USB MIDI readiness, CLI diagnose, docs en traceability tests falen.</x:v>
       </x:c>
       <x:c r="L8" s="36" t="str">
-        <x:v>USB MIDI input adapter en hardware smoke test.</x:v>
+        <x:v>UsbMidiHardwareInputAdapter en midi diagnose-usb-input.</x:v>
       </x:c>
       <x:c r="M8" s="36" t="str">
         <x:v>US-019, US-024</x:v>
       </x:c>
       <x:c r="N8" s="38" t="str">
-        <x:v>Eerste fysieke controller.</x:v>
+        <x:v>Wacht op handmatige hardwaretest met minimaal een echt USB MIDI input device.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85e8499c63484c86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re24dfe031d474f29"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Update US-022 midi test procedure
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rb2c45696a1be4a81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R21f0849afc174914"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Re7011d3f7fd34734"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rcf202a436607413b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R35dcd1905ac144a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rf2a3d55a459f4585"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R121e6192a5a0475c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Re479b3e859b94bee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b8a862be2d54ef1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33c96d0393134dde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1793,19 +1793,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J8" s="36" t="str">
-        <x:v>Generieke USB MIDI inputdiagnose werkt voor KeyLab, Fishman TriplePlay, M-Vave en andere inputdevices.</x:v>
+        <x:v>Generieke USB MIDI inputdiagnose werkt na list-devices en expliciete device/default keuze.</x:v>
       </x:c>
       <x:c r="K8" s="36" t="str">
-        <x:v>USB MIDI readiness, CLI diagnose, docs en traceability tests falen.</x:v>
+        <x:v>USB MIDI readiness, CLI guidance, docs en traceability tests falen.</x:v>
       </x:c>
       <x:c r="L8" s="36" t="str">
-        <x:v>UsbMidiHardwareInputAdapter en midi diagnose-usb-input.</x:v>
+        <x:v>UsbMidiHardwareInputAdapter, midi diagnose-usb-input en scan-failure guidance.</x:v>
       </x:c>
       <x:c r="M8" s="36" t="str">
         <x:v>US-019, US-024</x:v>
       </x:c>
       <x:c r="N8" s="38" t="str">
-        <x:v>Wacht op handmatige hardwaretest met minimaal een echt USB MIDI input device.</x:v>
+        <x:v>Wacht op hardwaretest; noteer KodeklopperM4/MuziekM4, Logic-visible devices en gekozen/default device.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re24dfe031d474f29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1c31468b8ff4c31"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Record US-022 midi scan test result
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R35dcd1905ac144a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rf2a3d55a459f4585"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R121e6192a5a0475c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Re479b3e859b94bee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Ra9c61e9c9e7b4703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Reb07a06db92e471a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R7caeeaf9d33b4cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R93797f6c15d84ee8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33c96d0393134dde"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb6e9e33dadc435a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1805,7 +1805,7 @@
         <x:v>US-019, US-024</x:v>
       </x:c>
       <x:c r="N8" s="38" t="str">
-        <x:v>Wacht op hardwaretest; noteer KodeklopperM4/MuziekM4, Logic-visible devices en gekozen/default device.</x:v>
+        <x:v>KodeklopperM4 test: Logic toont devices, Python backend scan faalt; wacht op gekozen/default device of MuziekM4 test.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1c31468b8ff4c31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8697cf8368be45cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Diagnose US-022 midi backend blocker
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Ra9c61e9c9e7b4703"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Reb07a06db92e471a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R7caeeaf9d33b4cbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R93797f6c15d84ee8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rcab8b1ab4a1044bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R3f85204989ba46a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R15f8de97fc714f16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R2948a80abe7f4434"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb6e9e33dadc435a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8d88d9fab674f87"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1778,7 +1778,7 @@
         <x:v>USB MIDI Hardware Input</x:v>
       </x:c>
       <x:c r="E8" s="36" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="F8" s="36" t="str">
         <x:v>Must</x:v>
@@ -1796,16 +1796,16 @@
         <x:v>Generieke USB MIDI inputdiagnose werkt na list-devices en expliciete device/default keuze.</x:v>
       </x:c>
       <x:c r="K8" s="36" t="str">
-        <x:v>USB MIDI readiness, CLI guidance, docs en traceability tests falen.</x:v>
+        <x:v>Hardware MIDI test faalt wanneer Python geen devices scant terwijl Logic devices toont.</x:v>
       </x:c>
       <x:c r="L8" s="36" t="str">
-        <x:v>UsbMidiHardwareInputAdapter, midi diagnose-usb-input en scan-failure guidance.</x:v>
+        <x:v>Backenddetails, BLOCKER output en tests/test_hardware_midi.py voor echte device scan.</x:v>
       </x:c>
       <x:c r="M8" s="36" t="str">
         <x:v>US-019, US-024</x:v>
       </x:c>
       <x:c r="N8" s="38" t="str">
-        <x:v>KodeklopperM4 test: Logic toont devices, Python backend scan faalt; wacht op gekozen/default device of MuziekM4 test.</x:v>
+        <x:v>Impediment: rtmidi package-conflict opgelost; resterend is CoreMIDI/RtMidi SIGABRT in MidiInCore::initialize (-10833), bevestigd door crashlogs.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8697cf8368be45cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eb2e341239d40b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete US-022 midi hardware discovery
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rcab8b1ab4a1044bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R3f85204989ba46a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R15f8de97fc714f16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R2948a80abe7f4434"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rf36f725f05b14def"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rd446fdd8848d40a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rd3eaa40e1c6f44af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R7a3df17e0f464902"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8d88d9fab674f87"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc8cd6b0f5394def"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1778,7 +1778,7 @@
         <x:v>USB MIDI Hardware Input</x:v>
       </x:c>
       <x:c r="E8" s="36" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F8" s="36" t="str">
         <x:v>Must</x:v>
@@ -1805,7 +1805,7 @@
         <x:v>US-019, US-024</x:v>
       </x:c>
       <x:c r="N8" s="38" t="str">
-        <x:v>Impediment: rtmidi package-conflict opgelost; resterend is CoreMIDI/RtMidi SIGABRT in MidiInCore::initialize (-10833), bevestigd door crashlogs.</x:v>
+        <x:v>Klanttest geslaagd op KodeklopperM4: MIDI input/output devices gelist, inclusief Scarlett 8i6 USB, SMK-37 Pro_BLE en SN76489 CircuitPython ESP32 S2.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eb2e341239d40b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R962e1239288a428b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete US-023 studio midi routing matrix
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rf36f725f05b14def"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rd446fdd8848d40a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rd3eaa40e1c6f44af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R7a3df17e0f464902"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rca32c664e2924a2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R7af38d97886842f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rf5f573def5ba4477"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R1b1efb0ee9204487"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc8cd6b0f5394def"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75f247f7311c4335"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1822,7 +1822,7 @@
         <x:v>Studio MIDI Routing Integratietest</x:v>
       </x:c>
       <x:c r="E9" s="36" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F9" s="36" t="str">
         <x:v>Should</x:v>
@@ -1837,19 +1837,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J9" s="36" t="str">
-        <x:v>Testmatrix dekt RaspiMidiHub, fysieke MIDI hub, MiniFreak en KeyLab Mk3.</x:v>
+        <x:v>Testmatrix dekt DAW bus, USB MIDI, controllers, guitar MIDI, synth hardware, CircuitPython/ESP32, Windows en Raspberry Pi.</x:v>
       </x:c>
       <x:c r="K9" s="36" t="str">
         <x:v>Integratietestplan ontbreekt.</x:v>
       </x:c>
       <x:c r="L9" s="36" t="str">
-        <x:v>Routing testmatrix en testnotities.</x:v>
+        <x:v>Routing matrix, host snapshots en placeholder-regel voor device-namen.</x:v>
       </x:c>
       <x:c r="M9" s="36" t="str">
         <x:v>US-022</x:v>
       </x:c>
       <x:c r="N9" s="38" t="str">
-        <x:v>Studio-opstelling expliciet documenteren.</x:v>
+        <x:v>docs/studio_midi_routing_integration_v0.1.0.md legt KodeklopperM4 en MuziekM4 snapshots vast als testdata, niet als code constants.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R962e1239288a428b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99261b9e54e64776"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete US-024 midi note event mapping
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rca32c664e2924a2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R7af38d97886842f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rf5f573def5ba4477"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R1b1efb0ee9204487"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R8b57f48a291f475f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rb85ece45c5ff4acd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R22831891be204164"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rbe1471fb8a7e4f71"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75f247f7311c4335"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebf5c6e6dfa34af7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1866,7 +1866,7 @@
         <x:v>MIDI Naar NoteEvent Mapping</x:v>
       </x:c>
       <x:c r="E10" s="36" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F10" s="36" t="str">
         <x:v>Must</x:v>
@@ -1881,19 +1881,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J10" s="36" t="str">
-        <x:v>MIDI note on/off wordt correct naar NoteEvent gemapt.</x:v>
+        <x:v>MIDI note on/off wordt correct naar NoteEvent gemapt, inclusief channel en genormaliseerde velocity.</x:v>
       </x:c>
       <x:c r="K10" s="36" t="str">
-        <x:v>Mapper tests falen voor note number, channel en velocity.</x:v>
+        <x:v>Mapper tests falen voor note number, channel, velocity, velocity-zero note-off en ontbrekende note-off.</x:v>
       </x:c>
       <x:c r="L10" s="36" t="str">
-        <x:v>MidiToNoteEventMapper class.</x:v>
+        <x:v>MidiToNoteEventMapper class en VirtualMidiInputAdapter hergebruik van dezelfde mapper.</x:v>
       </x:c>
       <x:c r="M10" s="36" t="str">
         <x:v>US-006, US-019</x:v>
       </x:c>
       <x:c r="N10" s="38" t="str">
-        <x:v>Houdt Sprint 1 engine herbruikbaar.</x:v>
+        <x:v>pytest groen: note number 60 -&gt; C4, channels blijven gescheiden, default duration werkt en docs/traceability zijn bijgewerkt.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99261b9e54e64776"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44ab1dd6f104443b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete US-025 midi device selection
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R8b57f48a291f475f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rb85ece45c5ff4acd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R22831891be204164"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rbe1471fb8a7e4f71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R74aa2f94d99a4f64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Ree1aef70a43145ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R46b24d14a0cf4402"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R01221822e6b44032"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebf5c6e6dfa34af7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R634a3fc882b242c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1910,7 +1910,7 @@
         <x:v>MIDI Device Discovery En Default Selection</x:v>
       </x:c>
       <x:c r="E11" s="40" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F11" s="40" t="str">
         <x:v>Must</x:v>
@@ -1925,19 +1925,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J11" s="40" t="str">
-        <x:v>CLI scant MIDI devices veilig en kiest device via CLI of YAML default.</x:v>
+        <x:v>CLI scant MIDI devices veilig en kiest input via CLI naam, CLI identifier of YAML default.</x:v>
       </x:c>
       <x:c r="K11" s="40" t="str">
-        <x:v>Device discovery en config precedence tests falen.</x:v>
+        <x:v>Device discovery, identifier selectie, config precedence en missing-device tests falen.</x:v>
       </x:c>
       <x:c r="L11" s="40" t="str">
-        <x:v>MidiDeviceScanner met veilige macOS default en optionele --unsafe-rtmidi-scan.</x:v>
+        <x:v>MidiDeviceSelector, MidiDeviceSelection en midi list-devices flags --midi-device, --midi-device-id en --config.</x:v>
       </x:c>
       <x:c r="M11" s="40" t="str">
         <x:v>US-019, US-020, US-022</x:v>
       </x:c>
       <x:c r="N11" s="42" t="str">
-        <x:v>RtMidi/CoreMIDI crashrapporten voorkomen door native scan standaard uit te schakelen.</x:v>
+        <x:v>pytest groen: CLI wint van YAML, output devices worden niet als input geselecteerd, geen hardcoded MIDI device names.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1958,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44ab1dd6f104443b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13484e61f81f402c"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete US-026 live midi receive loop
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R74aa2f94d99a4f64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Ree1aef70a43145ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R46b24d14a0cf4402"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R01221822e6b44032"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rb4e9dc30f482457e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rf6c984072a744d2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R09ca7d1291734199"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rd7ab81a4ebec4312"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,8 +404,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N11"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N14"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R634a3fc882b242c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffc70bc4b1014cdf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1897,47 +1897,179 @@
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="39" t="str">
+      <x:c r="A11" s="35" t="str">
         <x:v>US-025</x:v>
       </x:c>
-      <x:c r="B11" s="40" t="str">
-        <x:v>Story</x:v>
-      </x:c>
-      <x:c r="C11" s="40" t="str">
+      <x:c r="B11" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C11" s="36" t="str">
         <x:v>Future MIDI En DAW Integratie</x:v>
       </x:c>
-      <x:c r="D11" s="40" t="str">
+      <x:c r="D11" s="36" t="str">
         <x:v>MIDI Device Discovery En Default Selection</x:v>
       </x:c>
-      <x:c r="E11" s="40" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="F11" s="40" t="str">
+      <x:c r="E11" s="36" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F11" s="36" t="str">
         <x:v>Must</x:v>
       </x:c>
-      <x:c r="G11" s="40" t="str">
+      <x:c r="G11" s="36" t="str">
         <x:v>Lead Developer</x:v>
       </x:c>
-      <x:c r="H11" s="41" t="n">
+      <x:c r="H11" s="37" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="I11" s="40" t="str">
+      <x:c r="I11" s="36" t="str">
         <x:v>Future</x:v>
       </x:c>
-      <x:c r="J11" s="40" t="str">
+      <x:c r="J11" s="36" t="str">
         <x:v>CLI scant MIDI devices veilig en kiest input via CLI naam, CLI identifier of YAML default.</x:v>
       </x:c>
-      <x:c r="K11" s="40" t="str">
+      <x:c r="K11" s="36" t="str">
         <x:v>Device discovery, identifier selectie, config precedence en missing-device tests falen.</x:v>
       </x:c>
-      <x:c r="L11" s="40" t="str">
+      <x:c r="L11" s="36" t="str">
         <x:v>MidiDeviceSelector, MidiDeviceSelection en midi list-devices flags --midi-device, --midi-device-id en --config.</x:v>
       </x:c>
-      <x:c r="M11" s="40" t="str">
+      <x:c r="M11" s="36" t="str">
         <x:v>US-019, US-020, US-022</x:v>
       </x:c>
-      <x:c r="N11" s="42" t="str">
+      <x:c r="N11" s="38" t="str">
         <x:v>pytest groen: CLI wint van YAML, output devices worden niet als input geselecteerd, geen hardcoded MIDI device names.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="35" t="str">
+        <x:v>US-026</x:v>
+      </x:c>
+      <x:c r="B12" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C12" s="36" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D12" s="36" t="str">
+        <x:v>Live MIDI Input Receive Loop</x:v>
+      </x:c>
+      <x:c r="E12" s="36" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F12" s="36" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="G12" s="36" t="str">
+        <x:v>Lead Developer</x:v>
+      </x:c>
+      <x:c r="H12" s="37" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I12" s="36" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J12" s="36" t="str">
+        <x:v>CLI luistert bounded naar gekozen MIDI input en mapped note messages naar NoteSequence.</x:v>
+      </x:c>
+      <x:c r="K12" s="36" t="str">
+        <x:v>Normalizer, fake receive backend en midi listen CLI tests falen.</x:v>
+      </x:c>
+      <x:c r="L12" s="36" t="str">
+        <x:v>MidiMessageNormalizer, LiveMidiInputReceiver, MidiInputReceiveSettings/Result en midi listen command.</x:v>
+      </x:c>
+      <x:c r="M12" s="36" t="str">
+        <x:v>US-024, US-025</x:v>
+      </x:c>
+      <x:c r="N12" s="38" t="str">
+        <x:v>pytest groen: fake backend ontvangt note_on/off, geen Logic virtual device en geen realtime audio-trigger.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="35" t="str">
+        <x:v>US-027</x:v>
+      </x:c>
+      <x:c r="B13" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C13" s="36" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D13" s="36" t="str">
+        <x:v>Virtual MIDI Port Voor Logic/DAW</x:v>
+      </x:c>
+      <x:c r="E13" s="36" t="str">
+        <x:v>To Do</x:v>
+      </x:c>
+      <x:c r="F13" s="36" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="G13" s="36" t="str">
+        <x:v>Lead Developer</x:v>
+      </x:c>
+      <x:c r="H13" s="37" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I13" s="36" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J13" s="36" t="str">
+        <x:v>python-d1-synth kan later als virtual MIDI destination zichtbaar worden voor Logic/DAW.</x:v>
+      </x:c>
+      <x:c r="K13" s="36" t="str">
+        <x:v>Virtual port creation tests ontbreken.</x:v>
+      </x:c>
+      <x:c r="L13" s="36" t="str">
+        <x:v>Nog niet implementeren; eerst US-026 hardwaretest en design review.</x:v>
+      </x:c>
+      <x:c r="M13" s="36" t="str">
+        <x:v>US-026</x:v>
+      </x:c>
+      <x:c r="N13" s="38" t="str">
+        <x:v>Bewust uit US-026 gehouden om side quest scope creep te voorkomen.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="39" t="str">
+        <x:v>US-028</x:v>
+      </x:c>
+      <x:c r="B14" s="40" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C14" s="40" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D14" s="40" t="str">
+        <x:v>External MIDI Audio Trigger Integratie</x:v>
+      </x:c>
+      <x:c r="E14" s="40" t="str">
+        <x:v>To Do</x:v>
+      </x:c>
+      <x:c r="F14" s="40" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="G14" s="40" t="str">
+        <x:v>DSP Engineer</x:v>
+      </x:c>
+      <x:c r="H14" s="41" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I14" s="40" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J14" s="40" t="str">
+        <x:v>Ontvangen MIDI note events triggeren hoorbaar audio via de bestaande synth engine.</x:v>
+      </x:c>
+      <x:c r="K14" s="40" t="str">
+        <x:v>Live MIDI naar audio integration tests ontbreken.</x:v>
+      </x:c>
+      <x:c r="L14" s="40" t="str">
+        <x:v>Nog niet implementeren; vereist receive-loop validatie en audio scheduling ontwerp.</x:v>
+      </x:c>
+      <x:c r="M14" s="40" t="str">
+        <x:v>US-026, US-027</x:v>
+      </x:c>
+      <x:c r="N14" s="42" t="str">
+        <x:v>Bewust uit US-026 gehouden; dit is de eerste live speelbare MIDI-audio story.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1958,7 +2090,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13484e61f81f402c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bf9b845f9af4d78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2106,8 +2238,8 @@
         <x:v>Future MIDI/DAW Stories</x:v>
       </x:c>
       <x:c r="B9" s="44" t="n">
-        <x:f>COUNTA('Future MIDI DAW'!A5:A11)</x:f>
-        <x:v>7</x:v>
+        <x:f>COUNTA('Future MIDI DAW'!A5:A14)</x:f>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2115,8 +2247,8 @@
         <x:v>Future MIDI/DAW Points</x:v>
       </x:c>
       <x:c r="B10" s="44" t="n">
-        <x:f>SUM('Future MIDI DAW'!H5:H11)</x:f>
-        <x:v>26</x:v>
+        <x:f>SUM('Future MIDI DAW'!H5:H14)</x:f>
+        <x:v>44</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
Document US-026 hardware midi validation
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rb4e9dc30f482457e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rf6c984072a744d2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R09ca7d1291734199"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rd7ab81a4ebec4312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R688bd8f910e74445"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rd54559f330b948a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R46c89a6257c541f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rac9528444f554693"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffc70bc4b1014cdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb193309b53214dd3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1981,7 +1981,7 @@
         <x:v>US-024, US-025</x:v>
       </x:c>
       <x:c r="N12" s="38" t="str">
-        <x:v>pytest groen: fake backend ontvangt note_on/off, geen Logic virtual device en geen realtime audio-trigger.</x:v>
+        <x:v>pytest groen en hardwaretest geslaagd op KodeklopperM4: SMK-37 Pro_BLE Bluetooth via naamfragment en input:7 ontving echte MIDI note messages.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -2090,7 +2090,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bf9b845f9af4d78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfba10fb659144c66"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete US-027 virtual MIDI port workflow
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R688bd8f910e74445"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rd54559f330b948a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R46c89a6257c541f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rac9528444f554693"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R18b6be3c201f4ab2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R64824e364a034cf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R84bd7b40b3b24e3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Raec5738261c54167"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb193309b53214dd3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcb897ff4a4a4fe3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1998,7 +1998,7 @@
         <x:v>Virtual MIDI Port Voor Logic/DAW</x:v>
       </x:c>
       <x:c r="E13" s="36" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="F13" s="36" t="str">
         <x:v>Should</x:v>
@@ -2013,19 +2013,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J13" s="36" t="str">
-        <x:v>python-d1-synth kan later als virtual MIDI destination zichtbaar worden voor Logic/DAW.</x:v>
+        <x:v>python-d1-synth kan bounded als virtual MIDI destination zichtbaar worden voor Logic/DAW.</x:v>
       </x:c>
       <x:c r="K13" s="36" t="str">
-        <x:v>Virtual port creation tests ontbreken.</x:v>
+        <x:v>Logic Pro 12.3 handmatige zichtbaarheidstest moet nog door klant bevestigd worden.</x:v>
       </x:c>
       <x:c r="L13" s="36" t="str">
-        <x:v>Nog niet implementeren; eerst US-026 hardwaretest en design review.</x:v>
+        <x:v>VirtualMidiPortManager, MidoVirtualMidiPortBackend en midi virtual-port command met fake-backend tests.</x:v>
       </x:c>
       <x:c r="M13" s="36" t="str">
         <x:v>US-026</x:v>
       </x:c>
       <x:c r="N13" s="38" t="str">
-        <x:v>Bewust uit US-026 gehouden om side quest scope creep te voorkomen.</x:v>
+        <x:v>pytest groen; story blijft In Review tot Logic Pro de destination python-d1-synth toont of een blocker is vastgelegd.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -2090,7 +2090,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfba10fb659144c66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95ea2015ef2444cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Record US-027 Logic validation
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R18b6be3c201f4ab2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R64824e364a034cf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R84bd7b40b3b24e3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Raec5738261c54167"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R596439a175e241f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rb300b319efe24343"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R1109d8a1259a4f53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Re868aa4f311e4b24"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcb897ff4a4a4fe3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b89e40c494549c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1998,7 +1998,7 @@
         <x:v>Virtual MIDI Port Voor Logic/DAW</x:v>
       </x:c>
       <x:c r="E13" s="36" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F13" s="36" t="str">
         <x:v>Should</x:v>
@@ -2016,7 +2016,7 @@
         <x:v>python-d1-synth kan bounded als virtual MIDI destination zichtbaar worden voor Logic/DAW.</x:v>
       </x:c>
       <x:c r="K13" s="36" t="str">
-        <x:v>Logic Pro 12.3 handmatige zichtbaarheidstest moet nog door klant bevestigd worden.</x:v>
+        <x:v>Logic Pro 12.3 moet python-d1-synth tonen als External MIDI destination.</x:v>
       </x:c>
       <x:c r="L13" s="36" t="str">
         <x:v>VirtualMidiPortManager, MidoVirtualMidiPortBackend en midi virtual-port command met fake-backend tests.</x:v>
@@ -2025,7 +2025,7 @@
         <x:v>US-026</x:v>
       </x:c>
       <x:c r="N13" s="38" t="str">
-        <x:v>pytest groen; story blijft In Review tot Logic Pro de destination python-d1-synth toont of een blocker is vastgelegd.</x:v>
+        <x:v>Klanttest geslaagd op 2026-07-10 19:25: python-d1-synth zichtbaar als External MIDI destination; niet als Software Instrument is verwacht en buiten US-027.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -2090,7 +2090,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95ea2015ef2444cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raba192b0995745f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add US-028 external MIDI audio trigger
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R596439a175e241f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rb300b319efe24343"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R1109d8a1259a4f53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Re868aa4f311e4b24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rbd3f8f0818c44164"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R5caec341af2c49ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R52cf400f07a94980"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R5aa096d07a10488e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b89e40c494549c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ac11f9c09fe4ba9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2042,7 +2042,7 @@
         <x:v>External MIDI Audio Trigger Integratie</x:v>
       </x:c>
       <x:c r="E14" s="40" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="F14" s="40" t="str">
         <x:v>Must</x:v>
@@ -2060,16 +2060,16 @@
         <x:v>Ontvangen MIDI note events triggeren hoorbaar audio via de bestaande synth engine.</x:v>
       </x:c>
       <x:c r="K14" s="40" t="str">
-        <x:v>Live MIDI naar audio integration tests ontbreken.</x:v>
+        <x:v>MidiAudioTrigger en midi play-live tests falen totdat fake MIDI naar fake audio werkt.</x:v>
       </x:c>
       <x:c r="L14" s="40" t="str">
-        <x:v>Nog niet implementeren; vereist receive-loop validatie en audio scheduling ontwerp.</x:v>
+        <x:v>MidiAudioTriggerSettings/Result, MidiAudioTrigger en midi play-live command met fake MIDI en fake audio tests.</x:v>
       </x:c>
       <x:c r="M14" s="40" t="str">
         <x:v>US-026, US-027</x:v>
       </x:c>
       <x:c r="N14" s="42" t="str">
-        <x:v>Bewust uit US-026 gehouden; dit is de eerste live speelbare MIDI-audio story.</x:v>
+        <x:v>pytest groen; story blijft In Review tot klant hoorbare hardwaretest op Mac/Scarlett bevestigt.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2090,7 +2090,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raba192b0995745f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2d0473766964c96"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Record US-028 hardware validation
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rbd3f8f0818c44164"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R5caec341af2c49ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R52cf400f07a94980"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R5aa096d07a10488e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Re8a7154dfa5247dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Re50ad571f9bf4d78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R380936565e544eff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rf9628d7cb8e440f6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ac11f9c09fe4ba9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re29e35e0bfbf43dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2042,7 +2042,7 @@
         <x:v>External MIDI Audio Trigger Integratie</x:v>
       </x:c>
       <x:c r="E14" s="40" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F14" s="40" t="str">
         <x:v>Must</x:v>
@@ -2069,7 +2069,7 @@
         <x:v>US-026, US-027</x:v>
       </x:c>
       <x:c r="N14" s="42" t="str">
-        <x:v>pytest groen; story blijft In Review tot klant hoorbare hardwaretest op Mac/Scarlett bevestigt.</x:v>
+        <x:v>Klanttest geslaagd op KodeklopperM4: SMK-37 Pro_BLE Bluetooth speelde hoorbaar stereo audio via Scarlett 8i6 USB; Logic observatie buiten US-028.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2090,7 +2090,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2d0473766964c96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R531d9d6439204706"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add US-029 virtual MIDI audio trigger
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Re8a7154dfa5247dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Re50ad571f9bf4d78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R380936565e544eff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rf9628d7cb8e440f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R3003dde6147846da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R9b544f1a620045b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R4e906ee0bb1d4499"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rff05d0e6425c45ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,8 +404,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N14"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N15"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re29e35e0bfbf43dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra94db5a4db394d91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2029,47 +2029,91 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="39" t="str">
+      <x:c r="A14" s="35" t="str">
         <x:v>US-028</x:v>
       </x:c>
-      <x:c r="B14" s="40" t="str">
-        <x:v>Story</x:v>
-      </x:c>
-      <x:c r="C14" s="40" t="str">
+      <x:c r="B14" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C14" s="36" t="str">
         <x:v>Future MIDI En DAW Integratie</x:v>
       </x:c>
-      <x:c r="D14" s="40" t="str">
+      <x:c r="D14" s="36" t="str">
         <x:v>External MIDI Audio Trigger Integratie</x:v>
       </x:c>
-      <x:c r="E14" s="40" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="F14" s="40" t="str">
+      <x:c r="E14" s="36" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F14" s="36" t="str">
         <x:v>Must</x:v>
       </x:c>
-      <x:c r="G14" s="40" t="str">
+      <x:c r="G14" s="36" t="str">
         <x:v>DSP Engineer</x:v>
       </x:c>
-      <x:c r="H14" s="41" t="n">
+      <x:c r="H14" s="37" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="I14" s="40" t="str">
+      <x:c r="I14" s="36" t="str">
         <x:v>Future</x:v>
       </x:c>
-      <x:c r="J14" s="40" t="str">
+      <x:c r="J14" s="36" t="str">
         <x:v>Ontvangen MIDI note events triggeren hoorbaar audio via de bestaande synth engine.</x:v>
       </x:c>
-      <x:c r="K14" s="40" t="str">
+      <x:c r="K14" s="36" t="str">
         <x:v>MidiAudioTrigger en midi play-live tests falen totdat fake MIDI naar fake audio werkt.</x:v>
       </x:c>
-      <x:c r="L14" s="40" t="str">
+      <x:c r="L14" s="36" t="str">
         <x:v>MidiAudioTriggerSettings/Result, MidiAudioTrigger en midi play-live command met fake MIDI en fake audio tests.</x:v>
       </x:c>
-      <x:c r="M14" s="40" t="str">
+      <x:c r="M14" s="36" t="str">
         <x:v>US-026, US-027</x:v>
       </x:c>
-      <x:c r="N14" s="42" t="str">
+      <x:c r="N14" s="38" t="str">
         <x:v>Klanttest geslaagd op KodeklopperM4: SMK-37 Pro_BLE Bluetooth speelde hoorbaar stereo audio via Scarlett 8i6 USB; Logic observatie buiten US-028.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="39" t="str">
+        <x:v>US-029</x:v>
+      </x:c>
+      <x:c r="B15" s="40" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C15" s="40" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D15" s="40" t="str">
+        <x:v>Logic/DAW Virtual MIDI Naar Audio Trigger</x:v>
+      </x:c>
+      <x:c r="E15" s="40" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="F15" s="40" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="G15" s="40" t="str">
+        <x:v>DSP Engineer</x:v>
+      </x:c>
+      <x:c r="H15" s="41" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I15" s="40" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J15" s="40" t="str">
+        <x:v>Logic/DAW stuurt MIDI naar virtual port en python-d1-synth speelt hoorbare audio.</x:v>
+      </x:c>
+      <x:c r="K15" s="40" t="str">
+        <x:v>Virtual MIDI audio trigger en CLI play-virtual tests falen totdat fake virtual MIDI naar fake audio werkt.</x:v>
+      </x:c>
+      <x:c r="L15" s="40" t="str">
+        <x:v>MidoVirtualMidiInputBackend, VirtualMidiAudioTriggerSettings/Result, VirtualMidiAudioTrigger en midi play-virtual command.</x:v>
+      </x:c>
+      <x:c r="M15" s="40" t="str">
+        <x:v>US-027, US-028</x:v>
+      </x:c>
+      <x:c r="N15" s="42" t="str">
+        <x:v>pytest groen; handmatige Logic Pro test pauzeert bij klant.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2090,7 +2134,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R531d9d6439204706"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4943a5f3df2347ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2238,8 +2282,8 @@
         <x:v>Future MIDI/DAW Stories</x:v>
       </x:c>
       <x:c r="B9" s="44" t="n">
-        <x:f>COUNTA('Future MIDI DAW'!A5:A14)</x:f>
-        <x:v>10</x:v>
+        <x:f>COUNTA('Future MIDI DAW'!A5:A15)</x:f>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2247,8 +2291,8 @@
         <x:v>Future MIDI/DAW Points</x:v>
       </x:c>
       <x:c r="B10" s="44" t="n">
-        <x:f>SUM('Future MIDI DAW'!H5:H14)</x:f>
-        <x:v>44</x:v>
+        <x:f>SUM('Future MIDI DAW'!H5:H15)</x:f>
+        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
Record US-029 validation and lessons learned
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R3003dde6147846da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R9b544f1a620045b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R4e906ee0bb1d4499"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rff05d0e6425c45ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rd706125f091a4e55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Ra6f54b121b3247fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rbe146c6cdae443d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R7130de581e194d0e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra94db5a4db394d91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70a889afef7946fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2086,7 +2086,7 @@
         <x:v>Logic/DAW Virtual MIDI Naar Audio Trigger</x:v>
       </x:c>
       <x:c r="E15" s="40" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F15" s="40" t="str">
         <x:v>Must</x:v>
@@ -2113,7 +2113,7 @@
         <x:v>US-027, US-028</x:v>
       </x:c>
       <x:c r="N15" s="42" t="str">
-        <x:v>pytest groen; handmatige Logic Pro test pauzeert bij klant.</x:v>
+        <x:v>Klanttest geslaagd: Logic MIDI region speelde hoorbaar geluid; Python ontving note_on:60 velocity=50 channel=1 via python-d1-synth.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2134,7 +2134,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4943a5f3df2347ed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R568759e4b514441c"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add US-030 multi-note Logic playback
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rd706125f091a4e55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Ra6f54b121b3247fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rbe146c6cdae443d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R7130de581e194d0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rc7455d923f744786"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rf96c06a72e2d4906"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R8be9b46515ad49a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rfe58f0db65da405c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,8 +404,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N15"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N16"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70a889afef7946fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bed6dab9e8e489b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2073,47 +2073,91 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
-      <x:c r="A15" s="39" t="str">
+      <x:c r="A15" s="35" t="str">
         <x:v>US-029</x:v>
       </x:c>
-      <x:c r="B15" s="40" t="str">
-        <x:v>Story</x:v>
-      </x:c>
-      <x:c r="C15" s="40" t="str">
+      <x:c r="B15" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C15" s="36" t="str">
         <x:v>Future MIDI En DAW Integratie</x:v>
       </x:c>
-      <x:c r="D15" s="40" t="str">
+      <x:c r="D15" s="36" t="str">
         <x:v>Logic/DAW Virtual MIDI Naar Audio Trigger</x:v>
       </x:c>
-      <x:c r="E15" s="40" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="F15" s="40" t="str">
+      <x:c r="E15" s="36" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F15" s="36" t="str">
         <x:v>Must</x:v>
       </x:c>
-      <x:c r="G15" s="40" t="str">
+      <x:c r="G15" s="36" t="str">
         <x:v>DSP Engineer</x:v>
       </x:c>
-      <x:c r="H15" s="41" t="n">
+      <x:c r="H15" s="37" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="I15" s="40" t="str">
+      <x:c r="I15" s="36" t="str">
         <x:v>Future</x:v>
       </x:c>
-      <x:c r="J15" s="40" t="str">
+      <x:c r="J15" s="36" t="str">
         <x:v>Logic/DAW stuurt MIDI naar virtual port en python-d1-synth speelt hoorbare audio.</x:v>
       </x:c>
-      <x:c r="K15" s="40" t="str">
+      <x:c r="K15" s="36" t="str">
         <x:v>Virtual MIDI audio trigger en CLI play-virtual tests falen totdat fake virtual MIDI naar fake audio werkt.</x:v>
       </x:c>
-      <x:c r="L15" s="40" t="str">
+      <x:c r="L15" s="36" t="str">
         <x:v>MidoVirtualMidiInputBackend, VirtualMidiAudioTriggerSettings/Result, VirtualMidiAudioTrigger en midi play-virtual command.</x:v>
       </x:c>
-      <x:c r="M15" s="40" t="str">
+      <x:c r="M15" s="36" t="str">
         <x:v>US-027, US-028</x:v>
       </x:c>
-      <x:c r="N15" s="42" t="str">
+      <x:c r="N15" s="38" t="str">
         <x:v>Klanttest geslaagd: Logic MIDI region speelde hoorbaar geluid; Python ontving note_on:60 velocity=50 channel=1 via python-d1-synth.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="39" t="str">
+        <x:v>US-030</x:v>
+      </x:c>
+      <x:c r="B16" s="40" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C16" s="40" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D16" s="40" t="str">
+        <x:v>Logic MIDI Region Multi-Note Playback</x:v>
+      </x:c>
+      <x:c r="E16" s="40" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="F16" s="40" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="G16" s="40" t="str">
+        <x:v>DSP Engineer</x:v>
+      </x:c>
+      <x:c r="H16" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I16" s="40" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J16" s="40" t="str">
+        <x:v>Korte Logic MIDI region met meerdere noten rendert als hoorbare batch.</x:v>
+      </x:c>
+      <x:c r="K16" s="40" t="str">
+        <x:v>Multi-note mapping, fallback timing en verbose sequence-output tests falen.</x:v>
+      </x:c>
+      <x:c r="L16" s="40" t="str">
+        <x:v>MidiMessageNormalizer fallback time, VirtualMidiAudioTriggerResult.played_events en CLI Rendered sequence events output.</x:v>
+      </x:c>
+      <x:c r="M16" s="40" t="str">
+        <x:v>US-029</x:v>
+      </x:c>
+      <x:c r="N16" s="42" t="str">
+        <x:v>Automatische tests groen; wacht op Product Owner Logic multi-note test.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2134,7 +2178,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R568759e4b514441c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rceb6b90212ad4163"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2282,8 +2326,8 @@
         <x:v>Future MIDI/DAW Stories</x:v>
       </x:c>
       <x:c r="B9" s="44" t="n">
-        <x:f>COUNTA('Future MIDI DAW'!A5:A15)</x:f>
-        <x:v>11</x:v>
+        <x:f>COUNTA('Future MIDI DAW'!A5:A16)</x:f>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2291,8 +2335,8 @@
         <x:v>Future MIDI/DAW Points</x:v>
       </x:c>
       <x:c r="B10" s="44" t="n">
-        <x:f>SUM('Future MIDI DAW'!H5:H15)</x:f>
-        <x:v>52</x:v>
+        <x:f>SUM('Future MIDI DAW'!H5:H16)</x:f>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
Mark US-030 multi-note playback done
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rc7455d923f744786"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rf96c06a72e2d4906"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R8be9b46515ad49a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rfe58f0db65da405c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R5eeb32f47c87470c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R9b7bd73ffae242c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rcf6e308babbe408a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R0bdb87ddaf2e4d2c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bed6dab9e8e489b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb202ced7f7b34176"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2130,7 +2130,7 @@
         <x:v>Logic MIDI Region Multi-Note Playback</x:v>
       </x:c>
       <x:c r="E16" s="40" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F16" s="40" t="str">
         <x:v>Must</x:v>
@@ -2157,7 +2157,7 @@
         <x:v>US-029</x:v>
       </x:c>
       <x:c r="N16" s="42" t="str">
-        <x:v>Automatische tests groen; wacht op Product Owner Logic multi-note test.</x:v>
+        <x:v>Klanttest geslaagd: Logic speelde 5 hoorbare MIDI-triggered note events; circa 2s delay is batch-scope en geen blocker.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2178,7 +2178,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rceb6b90212ad4163"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6ff7de533d54cb1"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add US-031 streaming MIDI playback
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R5eeb32f47c87470c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R9b7bd73ffae242c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rcf6e308babbe408a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R0bdb87ddaf2e4d2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R8cb8832d807848e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R6e776eedb79f42fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R6b2d4819b97d42a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R5ed3d1ffdc4c4a75"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,8 +404,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N16"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N17"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb202ced7f7b34176"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R592fcd03b4b94267"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2117,47 +2117,91 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="39" t="str">
+      <x:c r="A16" s="35" t="str">
         <x:v>US-030</x:v>
       </x:c>
-      <x:c r="B16" s="40" t="str">
-        <x:v>Story</x:v>
-      </x:c>
-      <x:c r="C16" s="40" t="str">
+      <x:c r="B16" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C16" s="36" t="str">
         <x:v>Future MIDI En DAW Integratie</x:v>
       </x:c>
-      <x:c r="D16" s="40" t="str">
+      <x:c r="D16" s="36" t="str">
         <x:v>Logic MIDI Region Multi-Note Playback</x:v>
       </x:c>
-      <x:c r="E16" s="40" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="F16" s="40" t="str">
+      <x:c r="E16" s="36" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F16" s="36" t="str">
         <x:v>Must</x:v>
       </x:c>
-      <x:c r="G16" s="40" t="str">
+      <x:c r="G16" s="36" t="str">
         <x:v>DSP Engineer</x:v>
       </x:c>
-      <x:c r="H16" s="41" t="n">
+      <x:c r="H16" s="37" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="I16" s="40" t="str">
+      <x:c r="I16" s="36" t="str">
         <x:v>Future</x:v>
       </x:c>
-      <x:c r="J16" s="40" t="str">
+      <x:c r="J16" s="36" t="str">
         <x:v>Korte Logic MIDI region met meerdere noten rendert als hoorbare batch.</x:v>
       </x:c>
-      <x:c r="K16" s="40" t="str">
+      <x:c r="K16" s="36" t="str">
         <x:v>Multi-note mapping, fallback timing en verbose sequence-output tests falen.</x:v>
       </x:c>
-      <x:c r="L16" s="40" t="str">
+      <x:c r="L16" s="36" t="str">
         <x:v>MidiMessageNormalizer fallback time, VirtualMidiAudioTriggerResult.played_events en CLI Rendered sequence events output.</x:v>
       </x:c>
-      <x:c r="M16" s="40" t="str">
+      <x:c r="M16" s="36" t="str">
         <x:v>US-029</x:v>
       </x:c>
-      <x:c r="N16" s="42" t="str">
+      <x:c r="N16" s="38" t="str">
         <x:v>Klanttest geslaagd: Logic speelde 5 hoorbare MIDI-triggered note events; circa 2s delay is batch-scope en geen blocker.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="39" t="str">
+        <x:v>US-031</x:v>
+      </x:c>
+      <x:c r="B17" s="40" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C17" s="40" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D17" s="40" t="str">
+        <x:v>Live/Streaming MIDI Playback Loop</x:v>
+      </x:c>
+      <x:c r="E17" s="40" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="F17" s="40" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="G17" s="40" t="str">
+        <x:v>DSP Engineer</x:v>
+      </x:c>
+      <x:c r="H17" s="41" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I17" s="40" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J17" s="40" t="str">
+        <x:v>Ontvangen note_on events spelen direct als korte audio buffers.</x:v>
+      </x:c>
+      <x:c r="K17" s="40" t="str">
+        <x:v>Streaming backend, per-note audio calls en play-stream CLI tests falen.</x:v>
+      </x:c>
+      <x:c r="L17" s="40" t="str">
+        <x:v>MidoStreamingVirtualMidiInputBackend, StreamingMidiAudioTrigger en midi play-stream command.</x:v>
+      </x:c>
+      <x:c r="M17" s="40" t="str">
+        <x:v>US-030</x:v>
+      </x:c>
+      <x:c r="N17" s="42" t="str">
+        <x:v>Automatische tests groen; wacht op Product Owner Logic streaming latency test.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2178,7 +2222,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6ff7de533d54cb1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94b376177aef4346"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2326,8 +2370,8 @@
         <x:v>Future MIDI/DAW Stories</x:v>
       </x:c>
       <x:c r="B9" s="44" t="n">
-        <x:f>COUNTA('Future MIDI DAW'!A5:A16)</x:f>
-        <x:v>12</x:v>
+        <x:f>COUNTA('Future MIDI DAW'!A5:A17)</x:f>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2335,8 +2379,8 @@
         <x:v>Future MIDI/DAW Points</x:v>
       </x:c>
       <x:c r="B10" s="44" t="n">
-        <x:f>SUM('Future MIDI DAW'!H5:H16)</x:f>
-        <x:v>57</x:v>
+        <x:f>SUM('Future MIDI DAW'!H5:H17)</x:f>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
Mark US-031 done and plan MIDI roadmap
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R8cb8832d807848e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R6e776eedb79f42fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R6b2d4819b97d42a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R5ed3d1ffdc4c4a75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R2472fffd4f9d4086"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Ra7cf4f7ad0fe494b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rc31edc09912044b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rd70337b8872f4533"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,8 +404,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N17"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N22"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R592fcd03b4b94267"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R191ba44dfef34a3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2161,47 +2161,267 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
-      <x:c r="A17" s="39" t="str">
+      <x:c r="A17" s="35" t="str">
         <x:v>US-031</x:v>
       </x:c>
-      <x:c r="B17" s="40" t="str">
-        <x:v>Story</x:v>
-      </x:c>
-      <x:c r="C17" s="40" t="str">
+      <x:c r="B17" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C17" s="36" t="str">
         <x:v>Future MIDI En DAW Integratie</x:v>
       </x:c>
-      <x:c r="D17" s="40" t="str">
+      <x:c r="D17" s="36" t="str">
         <x:v>Live/Streaming MIDI Playback Loop</x:v>
       </x:c>
-      <x:c r="E17" s="40" t="str">
-        <x:v>In Review</x:v>
-      </x:c>
-      <x:c r="F17" s="40" t="str">
-        <x:v>Must</x:v>
-      </x:c>
-      <x:c r="G17" s="40" t="str">
+      <x:c r="E17" s="36" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F17" s="36" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="G17" s="36" t="str">
         <x:v>DSP Engineer</x:v>
       </x:c>
-      <x:c r="H17" s="41" t="n">
+      <x:c r="H17" s="37" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="I17" s="40" t="str">
+      <x:c r="I17" s="36" t="str">
         <x:v>Future</x:v>
       </x:c>
-      <x:c r="J17" s="40" t="str">
+      <x:c r="J17" s="36" t="str">
         <x:v>Ontvangen note_on events spelen direct als korte audio buffers.</x:v>
       </x:c>
-      <x:c r="K17" s="40" t="str">
+      <x:c r="K17" s="36" t="str">
         <x:v>Streaming backend, per-note audio calls en play-stream CLI tests falen.</x:v>
       </x:c>
-      <x:c r="L17" s="40" t="str">
+      <x:c r="L17" s="36" t="str">
         <x:v>MidoStreamingVirtualMidiInputBackend, StreamingMidiAudioTrigger en midi play-stream command.</x:v>
       </x:c>
-      <x:c r="M17" s="40" t="str">
+      <x:c r="M17" s="36" t="str">
         <x:v>US-030</x:v>
       </x:c>
-      <x:c r="N17" s="42" t="str">
-        <x:v>Automatische tests groen; wacht op Product Owner Logic streaming latency test.</x:v>
+      <x:c r="N17" s="38" t="str">
+        <x:v>Klanttest geslaagd: Logic streamde 18 hoorbare note events; dubbele events worden US-032.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="35" t="str">
+        <x:v>US-032</x:v>
+      </x:c>
+      <x:c r="B18" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C18" s="36" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D18" s="36" t="str">
+        <x:v>Duplicate MIDI Event Guard</x:v>
+      </x:c>
+      <x:c r="E18" s="36" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="F18" s="36" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="G18" s="36" t="str">
+        <x:v>DSP Engineer</x:v>
+      </x:c>
+      <x:c r="H18" s="37" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I18" s="36" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J18" s="36" t="str">
+        <x:v>Dubbele MIDI note events uit Logic/routing spelen niet dubbel hoorbaar af.</x:v>
+      </x:c>
+      <x:c r="K18" s="36" t="str">
+        <x:v>Dedup window en diagnostics tests falen.</x:v>
+      </x:c>
+      <x:c r="L18" s="36" t="str">
+        <x:v>Duplicate event guard voor streaming MIDI input.</x:v>
+      </x:c>
+      <x:c r="M18" s="36" t="str">
+        <x:v>US-031</x:v>
+      </x:c>
+      <x:c r="N18" s="38" t="str">
+        <x:v>Logische volgende story door dubbele note_on/note_off events in US-031 klanttest.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="35" t="str">
+        <x:v>US-033</x:v>
+      </x:c>
+      <x:c r="B19" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C19" s="36" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D19" s="36" t="str">
+        <x:v>Note Off Gated Voice Duration</x:v>
+      </x:c>
+      <x:c r="E19" s="36" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="F19" s="36" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="G19" s="36" t="str">
+        <x:v>DSP Engineer</x:v>
+      </x:c>
+      <x:c r="H19" s="37" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I19" s="36" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J19" s="36" t="str">
+        <x:v>Note-off bepaalt nootlengte in plaats van fixed note-duration.</x:v>
+      </x:c>
+      <x:c r="K19" s="36" t="str">
+        <x:v>Voice lifecycle tests falen.</x:v>
+      </x:c>
+      <x:c r="L19" s="36" t="str">
+        <x:v>Active voice state met note_on/note_off gating.</x:v>
+      </x:c>
+      <x:c r="M19" s="36" t="str">
+        <x:v>US-032</x:v>
+      </x:c>
+      <x:c r="N19" s="38" t="str">
+        <x:v>Voorbereiding voor sustain, polyfonie en latere envelopes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="35" t="str">
+        <x:v>US-034</x:v>
+      </x:c>
+      <x:c r="B20" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C20" s="36" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D20" s="36" t="str">
+        <x:v>Polyphonic Voice Mixer En Triads</x:v>
+      </x:c>
+      <x:c r="E20" s="36" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="F20" s="36" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="G20" s="36" t="str">
+        <x:v>DSP Engineer</x:v>
+      </x:c>
+      <x:c r="H20" s="37" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I20" s="36" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J20" s="36" t="str">
+        <x:v>Drie of meer gelijktijdige noten kunnen als triads hoorbaar worden gemixt.</x:v>
+      </x:c>
+      <x:c r="K20" s="36" t="str">
+        <x:v>Polyphonic mixer tests falen.</x:v>
+      </x:c>
+      <x:c r="L20" s="36" t="str">
+        <x:v>Meerdere actieve voices en clipping/level beheer.</x:v>
+      </x:c>
+      <x:c r="M20" s="36" t="str">
+        <x:v>US-033</x:v>
+      </x:c>
+      <x:c r="N20" s="38" t="str">
+        <x:v>Nodig voor akkoorden en later betere DAW playback.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="35" t="str">
+        <x:v>US-035</x:v>
+      </x:c>
+      <x:c r="B21" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C21" s="36" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D21" s="36" t="str">
+        <x:v>MIDI Pitch Bend Mapping En DSP</x:v>
+      </x:c>
+      <x:c r="E21" s="36" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="F21" s="36" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="G21" s="36" t="str">
+        <x:v>DSP Engineer</x:v>
+      </x:c>
+      <x:c r="H21" s="37" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I21" s="36" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J21" s="36" t="str">
+        <x:v>Pitch bend events buigen oscillatorfrequentie hoorbaar.</x:v>
+      </x:c>
+      <x:c r="K21" s="36" t="str">
+        <x:v>Pitch bend mapping en DSP tests falen.</x:v>
+      </x:c>
+      <x:c r="L21" s="36" t="str">
+        <x:v>Pitch bend parser plus frequentie-offset per channel/voice.</x:v>
+      </x:c>
+      <x:c r="M21" s="36" t="str">
+        <x:v>US-033, US-034</x:v>
+      </x:c>
+      <x:c r="N21" s="38" t="str">
+        <x:v>Pitch bend pas na betrouwbare voice state.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="39" t="str">
+        <x:v>US-036</x:v>
+      </x:c>
+      <x:c r="B22" s="40" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C22" s="40" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D22" s="40" t="str">
+        <x:v>MIDI Modulation CC1 Mapping En DSP</x:v>
+      </x:c>
+      <x:c r="E22" s="40" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="F22" s="40" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="G22" s="40" t="str">
+        <x:v>DSP Engineer</x:v>
+      </x:c>
+      <x:c r="H22" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I22" s="40" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J22" s="40" t="str">
+        <x:v>CC1 modulation stuurt een hoorbare synthparameter aan.</x:v>
+      </x:c>
+      <x:c r="K22" s="40" t="str">
+        <x:v>CC1 mapping tests falen.</x:v>
+      </x:c>
+      <x:c r="L22" s="40" t="str">
+        <x:v>Control change parser plus eenvoudige modulation target.</x:v>
+      </x:c>
+      <x:c r="M22" s="40" t="str">
+        <x:v>US-033, US-034</x:v>
+      </x:c>
+      <x:c r="N22" s="42" t="str">
+        <x:v>Eerste target later kiezen: vibrato of filter.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2222,7 +2442,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94b376177aef4346"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R365f60b2eb494a96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2370,8 +2590,8 @@
         <x:v>Future MIDI/DAW Stories</x:v>
       </x:c>
       <x:c r="B9" s="44" t="n">
-        <x:f>COUNTA('Future MIDI DAW'!A5:A17)</x:f>
-        <x:v>13</x:v>
+        <x:f>COUNTA('Future MIDI DAW'!A5:A22)</x:f>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2379,8 +2599,8 @@
         <x:v>Future MIDI/DAW Points</x:v>
       </x:c>
       <x:c r="B10" s="44" t="n">
-        <x:f>SUM('Future MIDI DAW'!H5:H17)</x:f>
-        <x:v>65</x:v>
+        <x:f>SUM('Future MIDI DAW'!H5:H22)</x:f>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
Add US-032 duplicate MIDI event guard
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R2472fffd4f9d4086"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Ra7cf4f7ad0fe494b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rc31edc09912044b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rd70337b8872f4533"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R8c3a34d2db1044e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rdb7d39979b364420"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R03596e08f3604637"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R80909f3e52f04739"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R191ba44dfef34a3c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9263505ddfc47c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2218,7 +2218,7 @@
         <x:v>Duplicate MIDI Event Guard</x:v>
       </x:c>
       <x:c r="E18" s="36" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="F18" s="36" t="str">
         <x:v>Must</x:v>
@@ -2233,19 +2233,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J18" s="36" t="str">
-        <x:v>Dubbele MIDI note events uit Logic/routing spelen niet dubbel hoorbaar af.</x:v>
+        <x:v>Dubbele MIDI note events uit Logic/routing spelen niet dubbel hoorbaar af, zonder simultane verschillende noten te onderdrukken.</x:v>
       </x:c>
       <x:c r="K18" s="36" t="str">
-        <x:v>Dedup window en diagnostics tests falen.</x:v>
+        <x:v>Dedup window, streaming duplicate suppression, CLI diagnostics en traceability tests falen.</x:v>
       </x:c>
       <x:c r="L18" s="36" t="str">
-        <x:v>Duplicate event guard voor streaming MIDI input.</x:v>
+        <x:v>DuplicateMidiEventGuard, --dedupe-window, suppressed_duplicate_count en docs/duplicate_midi_event_guard_v0.1.0.md.</x:v>
       </x:c>
       <x:c r="M18" s="36" t="str">
         <x:v>US-031</x:v>
       </x:c>
       <x:c r="N18" s="38" t="str">
-        <x:v>Logische volgende story door dubbele note_on/note_off events in US-031 klanttest.</x:v>
+        <x:v>In review: Logic/CoreMIDI echo-paren worden gefilterd; polyfonie, pitch bend en modulation blijven latere stories.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -2442,7 +2442,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R365f60b2eb494a96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb344039a32de44ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Mark US-032 duplicate MIDI guard done
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R8c3a34d2db1044e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rdb7d39979b364420"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R03596e08f3604637"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R80909f3e52f04739"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R37558de058fa42b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rc736e599763c4fce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R0270d17e55f74a59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Ra8e0cd13d7df44c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9263505ddfc47c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R743baddc5448432a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2218,7 +2218,7 @@
         <x:v>Duplicate MIDI Event Guard</x:v>
       </x:c>
       <x:c r="E18" s="36" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F18" s="36" t="str">
         <x:v>Must</x:v>
@@ -2245,7 +2245,7 @@
         <x:v>US-031</x:v>
       </x:c>
       <x:c r="N18" s="38" t="str">
-        <x:v>In review: Logic/CoreMIDI echo-paren worden gefilterd; polyfonie, pitch bend en modulation blijven latere stories.</x:v>
+        <x:v>Klanttest geslaagd: Logic/live playback hoorbaar; 6 note events gespeeld en 23 duplicate MIDI messages onderdrukt. Kleine latency blijft latere story.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -2442,7 +2442,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb344039a32de44ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cb3d19c30f84163"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add US-033 gated MIDI note duration
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R37558de058fa42b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rc736e599763c4fce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R0270d17e55f74a59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Ra8e0cd13d7df44c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R6c8065dcc6ef4493"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R05357698ee394b97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R04690355ccf14c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R4edddb12b47a4ba6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R743baddc5448432a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb30e7e863bd4382"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2262,7 +2262,7 @@
         <x:v>Note Off Gated Voice Duration</x:v>
       </x:c>
       <x:c r="E19" s="36" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="F19" s="36" t="str">
         <x:v>Must</x:v>
@@ -2277,19 +2277,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J19" s="36" t="str">
-        <x:v>Note-off bepaalt nootlengte in plaats van fixed note-duration.</x:v>
+        <x:v>Note-off bepaalt nootlengte in gated streaming mode in plaats van alleen fixed note-duration.</x:v>
       </x:c>
       <x:c r="K19" s="36" t="str">
-        <x:v>Voice lifecycle tests falen.</x:v>
+        <x:v>Voice mode, note_on/note_off duration, fallback duration, CLI diagnostics en traceability tests falen.</x:v>
       </x:c>
       <x:c r="L19" s="36" t="str">
-        <x:v>Active voice state met note_on/note_off gating.</x:v>
+        <x:v>StreamingVoiceMode, --voice-mode gated, active note state per MIDI key en Streamed note durations output.</x:v>
       </x:c>
       <x:c r="M19" s="36" t="str">
         <x:v>US-032</x:v>
       </x:c>
       <x:c r="N19" s="38" t="str">
-        <x:v>Voorbereiding voor sustain, polyfonie en latere envelopes.</x:v>
+        <x:v>In review: default fixed mode blijft bestaan; sustain, polyfonie, pitch bend en modulation blijven latere stories.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -2442,7 +2442,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cb3d19c30f84163"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b056717412f4023"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add US-035 sustained MIDI playback
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2093,7 +2093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="E20" s="36" t="inlineStr">
         <is>
-          <t>In Review</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F20" s="36" t="inlineStr">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="N20" s="38" t="inlineStr">
         <is>
-          <t>In review: triads/akkoorden klinken als polyphonic fixed/fallback buffers; sustained voices, pitch bend en modulation blijven latere stories.</t>
+          <t>Done: Product Owner hoorde akkoordachtige groepen met --chord-window 0.08; sustained voices blijven US-035.</t>
         </is>
       </c>
     </row>
@@ -3336,17 +3336,17 @@
       </c>
       <c r="D21" s="36" t="inlineStr">
         <is>
-          <t>MIDI Pitch Bend Mapping En DSP</t>
+          <t>Sustained Note Audio Engine</t>
         </is>
       </c>
       <c r="E21" s="36" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="F21" s="36" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t>Must</t>
         </is>
       </c>
       <c r="G21" s="36" t="inlineStr">
@@ -3355,7 +3355,7 @@
         </is>
       </c>
       <c r="H21" s="47" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I21" s="36" t="inlineStr">
         <is>
@@ -3364,27 +3364,27 @@
       </c>
       <c r="J21" s="36" t="inlineStr">
         <is>
-          <t>Pitch bend events buigen oscillatorfrequentie hoorbaar.</t>
+          <t>note_on start een streaming voice en note_off stopt die voice zodat vastgehouden noten hoorbaar aanhouden.</t>
         </is>
       </c>
       <c r="K21" s="36" t="inlineStr">
         <is>
-          <t>Pitch bend mapping en DSP tests falen.</t>
+          <t>Sustained audio player, voice lifecycle, CLI sustained mode en traceability tests falen.</t>
         </is>
       </c>
       <c r="L21" s="36" t="inlineStr">
         <is>
-          <t>Pitch bend parser plus frequentie-offset per channel/voice.</t>
+          <t>SoundDeviceSustainedAudioPlayer, SustainedAudioPlayerSettings, StreamingVoiceMode.SUSTAINED en --voice-mode sustained.</t>
         </is>
       </c>
       <c r="M21" s="36" t="inlineStr">
         <is>
-          <t>US-033, US-034</t>
+          <t>US-034</t>
         </is>
       </c>
       <c r="N21" s="38" t="inlineStr">
         <is>
-          <t>Pitch bend pas na betrouwbare voice state.</t>
+          <t>In review: sustained note-on/note-off lifecycle; sustain pedal, envelope release, pitch bend en modulation blijven latere stories.</t>
         </is>
       </c>
     </row>
@@ -3406,7 +3406,7 @@
       </c>
       <c r="D22" s="40" t="inlineStr">
         <is>
-          <t>MIDI Modulation CC1 Mapping En DSP</t>
+          <t>MIDI Pitch Bend Mapping En DSP</t>
         </is>
       </c>
       <c r="E22" s="40" t="inlineStr">
@@ -3434,25 +3434,95 @@
       </c>
       <c r="J22" s="40" t="inlineStr">
         <is>
+          <t>Pitch bend events buigen oscillatorfrequentie hoorbaar.</t>
+        </is>
+      </c>
+      <c r="K22" s="40" t="inlineStr">
+        <is>
+          <t>Pitch bend mapping en DSP tests falen.</t>
+        </is>
+      </c>
+      <c r="L22" s="40" t="inlineStr">
+        <is>
+          <t>Pitch bend parser plus frequentie-offset per channel/voice.</t>
+        </is>
+      </c>
+      <c r="M22" s="40" t="inlineStr">
+        <is>
+          <t>US-035</t>
+        </is>
+      </c>
+      <c r="N22" s="42" t="inlineStr">
+        <is>
+          <t>Pitch bend pas na betrouwbare sustained voice state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>US-037</t>
+        </is>
+      </c>
+      <c r="B23" s="40" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C23" s="40" t="inlineStr">
+        <is>
+          <t>Future MIDI En DAW Integratie</t>
+        </is>
+      </c>
+      <c r="D23" s="40" t="inlineStr">
+        <is>
+          <t>MIDI Modulation CC1 Mapping En DSP</t>
+        </is>
+      </c>
+      <c r="E23" s="40" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="F23" s="40" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G23" s="40" t="inlineStr">
+        <is>
+          <t>DSP Engineer</t>
+        </is>
+      </c>
+      <c r="H23" s="48" t="n">
+        <v>5</v>
+      </c>
+      <c r="I23" s="40" t="inlineStr">
+        <is>
+          <t>Future</t>
+        </is>
+      </c>
+      <c r="J23" s="40" t="inlineStr">
+        <is>
           <t>CC1 modulation stuurt een hoorbare synthparameter aan.</t>
         </is>
       </c>
-      <c r="K22" s="40" t="inlineStr">
+      <c r="K23" s="40" t="inlineStr">
         <is>
           <t>CC1 mapping tests falen.</t>
         </is>
       </c>
-      <c r="L22" s="40" t="inlineStr">
+      <c r="L23" s="40" t="inlineStr">
         <is>
           <t>Control change parser plus eenvoudige modulation target.</t>
         </is>
       </c>
-      <c r="M22" s="40" t="inlineStr">
-        <is>
-          <t>US-033, US-034</t>
-        </is>
-      </c>
-      <c r="N22" s="42" t="inlineStr">
+      <c r="M23" s="40" t="inlineStr">
+        <is>
+          <t>US-035, US-036</t>
+        </is>
+      </c>
+      <c r="N23" s="42" t="inlineStr">
         <is>
           <t>Eerste target later kiezen: vibrato of filter.</t>
         </is>

</xml_diff>

<commit_message>
Add US-036 MIDI pitch bend
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -3341,7 +3341,7 @@
       </c>
       <c r="E21" s="36" t="inlineStr">
         <is>
-          <t>In Review</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F21" s="36" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="N21" s="38" t="inlineStr">
         <is>
-          <t>In review: sustained note-on/note-off lifecycle; sustain pedal, envelope release, pitch bend en modulation blijven latere stories.</t>
+          <t>Done: Product Owner hoorde sustained playback; Total streamed audio frames: 575172.</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="E22" s="40" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In Review</t>
         </is>
       </c>
       <c r="F22" s="40" t="inlineStr">
@@ -3434,17 +3434,17 @@
       </c>
       <c r="J22" s="40" t="inlineStr">
         <is>
-          <t>Pitch bend events buigen oscillatorfrequentie hoorbaar.</t>
+          <t>Pitch bend events buigen actieve sustained voices per MIDI channel hoorbaar.</t>
         </is>
       </c>
       <c r="K22" s="40" t="inlineStr">
         <is>
-          <t>Pitch bend mapping en DSP tests falen.</t>
+          <t>Pitchwheel normalisatie, pitch bend mapper, sustained player bend en CLI diagnostics tests falen.</t>
         </is>
       </c>
       <c r="L22" s="40" t="inlineStr">
         <is>
-          <t>Pitch bend parser plus frequentie-offset per channel/voice.</t>
+          <t>MidiMessage pitch_bend, MidiPitchBendMapper, --pitch-bend-range en SoundDeviceSustainedAudioPlayer.pitch_bend.</t>
         </is>
       </c>
       <c r="M22" s="40" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="N22" s="42" t="inlineStr">
         <is>
-          <t>Pitch bend pas na betrouwbare sustained voice state.</t>
+          <t>In review: pitch bend per MIDI channel op actieve sustained voices; modulation/CC1 blijft US-037.</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="M23" s="40" t="inlineStr">
         <is>
-          <t>US-035, US-036</t>
+          <t>US-036</t>
         </is>
       </c>
       <c r="N23" s="42" t="inlineStr">

</xml_diff>

<commit_message>
Add US-037 MIDI modulation CC1
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R6e50d14fe0544399"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R61a57edea1544cf8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rd992ed95dcf8492e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R183d827bc1b6474f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R8d3df0ab0d0e47ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R66b71ba98d494a79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Reb11e8d03df04c03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R7dbf0a3fb478438e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R671167df69ad40bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a7ed73878d14264"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2394,7 +2394,7 @@
         <x:v>MIDI Pitch Bend Mapping En DSP</x:v>
       </x:c>
       <x:c r="E22" s="36" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="F22" s="36" t="str">
         <x:v>Should</x:v>
@@ -2421,7 +2421,7 @@
         <x:v>US-035</x:v>
       </x:c>
       <x:c r="N22" s="38" t="str">
-        <x:v>Impediment-001: SMK37/Logic kan note-on op channel 1 en pitch bend op channel 4 sturen; gebruik --pitch-bend-channel-mode omni.</x:v>
+        <x:v>Product Owner accepteerde hoorbare sustained playback, triads, korte/lange nootduur en nette Ctrl-C interrupt met --timeout 600.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
@@ -2438,7 +2438,7 @@
         <x:v>MIDI Modulation CC1 Mapping En DSP</x:v>
       </x:c>
       <x:c r="E23" s="40" t="str">
-        <x:v>Planned</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="F23" s="40" t="str">
         <x:v>Should</x:v>
@@ -2453,19 +2453,19 @@
         <x:v>Future</x:v>
       </x:c>
       <x:c r="J23" s="40" t="str">
-        <x:v>CC1 modulation stuurt een hoorbare synthparameter aan.</x:v>
+        <x:v>CC1 modulation stuurt eenvoudige vibrato-depth op sustained voices aan.</x:v>
       </x:c>
       <x:c r="K23" s="40" t="str">
-        <x:v>CC1 mapping tests falen.</x:v>
+        <x:v>CC1 normalisatie, modulation mapper, sustained player modulation en CLI diagnostics tests falen.</x:v>
       </x:c>
       <x:c r="L23" s="40" t="str">
-        <x:v>Control change parser plus eenvoudige modulation target.</x:v>
+        <x:v>MidiModulationMapper, control_change normalisatie, --modulation-vibrato-depth en --modulation-vibrato-rate.</x:v>
       </x:c>
       <x:c r="M23" s="40" t="str">
         <x:v>US-036</x:v>
       </x:c>
       <x:c r="N23" s="42" t="str">
-        <x:v>Eerste target later kiezen: vibrato of filter.</x:v>
+        <x:v>In review: CC1 control_change wordt gelogd als control_change:1:&lt;waarde&gt;:channel=&lt;n&gt; en stuurt vibrato-depth.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2486,7 +2486,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf927c07f35cd4ed8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1259369a63414943"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add US-038 performance mode
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R8d3df0ab0d0e47ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R66b71ba98d494a79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Reb11e8d03df04c03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R7dbf0a3fb478438e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R1b33aabb449e423b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R5748be4dcb664f20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R1442c775216a4f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Re62c81031d354fc8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,8 +404,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N23"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N24"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a7ed73878d14264"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R123b1c5ce683426e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2425,47 +2425,91 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
-      <x:c r="A23" s="39" t="str">
+      <x:c r="A23" s="35" t="str">
         <x:v>US-037</x:v>
       </x:c>
-      <x:c r="B23" s="40" t="str">
-        <x:v>Story</x:v>
-      </x:c>
-      <x:c r="C23" s="40" t="str">
+      <x:c r="B23" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C23" s="36" t="str">
         <x:v>Future MIDI En DAW Integratie</x:v>
       </x:c>
-      <x:c r="D23" s="40" t="str">
+      <x:c r="D23" s="36" t="str">
         <x:v>MIDI Modulation CC1 Mapping En DSP</x:v>
       </x:c>
-      <x:c r="E23" s="40" t="str">
+      <x:c r="E23" s="36" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F23" s="36" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="G23" s="36" t="str">
+        <x:v>DSP Engineer</x:v>
+      </x:c>
+      <x:c r="H23" s="37" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I23" s="36" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J23" s="36" t="str">
+        <x:v>CC1 modulation stuurt eenvoudige vibrato-depth op sustained voices aan.</x:v>
+      </x:c>
+      <x:c r="K23" s="36" t="str">
+        <x:v>CC1 normalisatie, modulation mapper, sustained player modulation en CLI diagnostics tests falen.</x:v>
+      </x:c>
+      <x:c r="L23" s="36" t="str">
+        <x:v>MidiModulationMapper, control_change normalisatie, --modulation-vibrato-depth en --modulation-vibrato-rate.</x:v>
+      </x:c>
+      <x:c r="M23" s="36" t="str">
+        <x:v>US-036</x:v>
+      </x:c>
+      <x:c r="N23" s="38" t="str">
+        <x:v>Klanttest geslaagd: pitch bend en CC1 modulation hoorbaar; interrupt-fix getest en akkoord.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="39" t="str">
+        <x:v>US-038</x:v>
+      </x:c>
+      <x:c r="B24" s="40" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C24" s="40" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D24" s="40" t="str">
+        <x:v>Performance Mode Until Interrupt</x:v>
+      </x:c>
+      <x:c r="E24" s="40" t="str">
         <x:v>In Review</x:v>
       </x:c>
-      <x:c r="F23" s="40" t="str">
-        <x:v>Should</x:v>
-      </x:c>
-      <x:c r="G23" s="40" t="str">
+      <x:c r="F24" s="40" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="G24" s="40" t="str">
         <x:v>DSP Engineer</x:v>
       </x:c>
-      <x:c r="H23" s="41" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="I23" s="40" t="str">
+      <x:c r="H24" s="41" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I24" s="40" t="str">
         <x:v>Future</x:v>
       </x:c>
-      <x:c r="J23" s="40" t="str">
-        <x:v>CC1 modulation stuurt eenvoudige vibrato-depth op sustained voices aan.</x:v>
-      </x:c>
-      <x:c r="K23" s="40" t="str">
-        <x:v>CC1 normalisatie, modulation mapper, sustained player modulation en CLI diagnostics tests falen.</x:v>
-      </x:c>
-      <x:c r="L23" s="40" t="str">
-        <x:v>MidiModulationMapper, control_change normalisatie, --modulation-vibrato-depth en --modulation-vibrato-rate.</x:v>
-      </x:c>
-      <x:c r="M23" s="40" t="str">
-        <x:v>US-036</x:v>
-      </x:c>
-      <x:c r="N23" s="42" t="str">
-        <x:v>In review: CC1 control_change wordt gelogd als control_change:1:&lt;waarde&gt;:channel=&lt;n&gt; en stuurt vibrato-depth.</x:v>
+      <x:c r="J24" s="40" t="str">
+        <x:v>play-stream kan als performance-run draaien tot Ctrl-C zonder korte testlimiet.</x:v>
+      </x:c>
+      <x:c r="K24" s="40" t="str">
+        <x:v>--until-interrupt, effective backend limits, Ctrl-C cleanup en CLI diagnostics tests falen.</x:v>
+      </x:c>
+      <x:c r="L24" s="40" t="str">
+        <x:v>StreamingMidiAudioTriggerSettings.run_until_interrupted, --until-interrupt en performance-mode README/docs.</x:v>
+      </x:c>
+      <x:c r="M24" s="40" t="str">
+        <x:v>US-037</x:v>
+      </x:c>
+      <x:c r="N24" s="42" t="str">
+        <x:v>In review: performance mode gebruikt praktische lange backend-limieten en meldt until_interrupt=true.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2486,7 +2530,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1259369a63414943"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b11224a7fba47f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2634,8 +2678,8 @@
         <x:v>Future MIDI/DAW Stories</x:v>
       </x:c>
       <x:c r="B9" s="44" t="n">
-        <x:f>COUNTA('Future MIDI DAW'!A5:A23)</x:f>
-        <x:v>19</x:v>
+        <x:f>COUNTA('Future MIDI DAW'!A5:A24)</x:f>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2643,8 +2687,8 @@
         <x:v>Future MIDI/DAW Points</x:v>
       </x:c>
       <x:c r="B10" s="44" t="n">
-        <x:f>SUM('Future MIDI DAW'!H5:H23)</x:f>
-        <x:v>104</x:v>
+        <x:f>SUM('Future MIDI DAW'!H5:H24)</x:f>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
Add US-039 sustain pedal CC64
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R1b33aabb449e423b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R5748be4dcb664f20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R1442c775216a4f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Re62c81031d354fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R5809faf442c54936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R3015f70e55d64399"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R4ce72be1e21e428c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R4dae8148ad784319"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,8 +404,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N24"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N25"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R123b1c5ce683426e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc887c1741cd45db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2469,47 +2469,91 @@
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
-      <x:c r="A24" s="39" t="str">
+      <x:c r="A24" s="35" t="str">
         <x:v>US-038</x:v>
       </x:c>
-      <x:c r="B24" s="40" t="str">
-        <x:v>Story</x:v>
-      </x:c>
-      <x:c r="C24" s="40" t="str">
+      <x:c r="B24" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C24" s="36" t="str">
         <x:v>Future MIDI En DAW Integratie</x:v>
       </x:c>
-      <x:c r="D24" s="40" t="str">
+      <x:c r="D24" s="36" t="str">
         <x:v>Performance Mode Until Interrupt</x:v>
       </x:c>
-      <x:c r="E24" s="40" t="str">
+      <x:c r="E24" s="36" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F24" s="36" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="G24" s="36" t="str">
+        <x:v>DSP Engineer</x:v>
+      </x:c>
+      <x:c r="H24" s="37" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I24" s="36" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J24" s="36" t="str">
+        <x:v>play-stream kan als performance-run draaien tot Ctrl-C zonder korte testlimiet.</x:v>
+      </x:c>
+      <x:c r="K24" s="36" t="str">
+        <x:v>--until-interrupt, effective backend limits, Ctrl-C cleanup en CLI diagnostics tests falen.</x:v>
+      </x:c>
+      <x:c r="L24" s="36" t="str">
+        <x:v>StreamingMidiAudioTriggerSettings.run_until_interrupted, --until-interrupt en performance-mode README/docs.</x:v>
+      </x:c>
+      <x:c r="M24" s="36" t="str">
+        <x:v>US-037</x:v>
+      </x:c>
+      <x:c r="N24" s="38" t="str">
+        <x:v>Klanttest geslaagd: performance mode met --until-interrupt werkt.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="39" t="str">
+        <x:v>US-039</x:v>
+      </x:c>
+      <x:c r="B25" s="40" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C25" s="40" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D25" s="40" t="str">
+        <x:v>Sustain Pedal CC64</x:v>
+      </x:c>
+      <x:c r="E25" s="40" t="str">
         <x:v>In Review</x:v>
       </x:c>
-      <x:c r="F24" s="40" t="str">
-        <x:v>Must</x:v>
-      </x:c>
-      <x:c r="G24" s="40" t="str">
+      <x:c r="F25" s="40" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="G25" s="40" t="str">
         <x:v>DSP Engineer</x:v>
       </x:c>
-      <x:c r="H24" s="41" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="I24" s="40" t="str">
+      <x:c r="H25" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I25" s="40" t="str">
         <x:v>Future</x:v>
       </x:c>
-      <x:c r="J24" s="40" t="str">
-        <x:v>play-stream kan als performance-run draaien tot Ctrl-C zonder korte testlimiet.</x:v>
-      </x:c>
-      <x:c r="K24" s="40" t="str">
-        <x:v>--until-interrupt, effective backend limits, Ctrl-C cleanup en CLI diagnostics tests falen.</x:v>
-      </x:c>
-      <x:c r="L24" s="40" t="str">
-        <x:v>StreamingMidiAudioTriggerSettings.run_until_interrupted, --until-interrupt en performance-mode README/docs.</x:v>
-      </x:c>
-      <x:c r="M24" s="40" t="str">
-        <x:v>US-037</x:v>
-      </x:c>
-      <x:c r="N24" s="42" t="str">
-        <x:v>In review: performance mode gebruikt praktische lange backend-limieten en meldt until_interrupt=true.</x:v>
+      <x:c r="J25" s="40" t="str">
+        <x:v>CC64 sustain pedal houdt released sustained voices vast tot pedal up.</x:v>
+      </x:c>
+      <x:c r="K25" s="40" t="str">
+        <x:v>CC64 down/up, held note release, CLI diagnostics en docs tests falen.</x:v>
+      </x:c>
+      <x:c r="L25" s="40" t="str">
+        <x:v>control_change:64 handling in sustained mode, pedal threshold 64 en docs/sustain_pedal_cc64_v0.1.0.md.</x:v>
+      </x:c>
+      <x:c r="M25" s="40" t="str">
+        <x:v>US-035, US-038</x:v>
+      </x:c>
+      <x:c r="N25" s="42" t="str">
+        <x:v>In review: CC64 64..127 is pedal down; 0..63 is pedal up.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2530,7 +2574,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b11224a7fba47f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09b68cf4f5864b89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2678,8 +2722,8 @@
         <x:v>Future MIDI/DAW Stories</x:v>
       </x:c>
       <x:c r="B9" s="44" t="n">
-        <x:f>COUNTA('Future MIDI DAW'!A5:A24)</x:f>
-        <x:v>20</x:v>
+        <x:f>COUNTA('Future MIDI DAW'!A5:A25)</x:f>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2687,8 +2731,8 @@
         <x:v>Future MIDI/DAW Points</x:v>
       </x:c>
       <x:c r="B10" s="44" t="n">
-        <x:f>SUM('Future MIDI DAW'!H5:H24)</x:f>
-        <x:v>107</x:v>
+        <x:f>SUM('Future MIDI DAW'!H5:H25)</x:f>
+        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
Add US-040 envelope release
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R0e9b73306b444edf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R8911218ca9364c7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R9dd532c6646f4a09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rb1f806adcd3040f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R3a30ea911d6e42b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R93679ac592a64c9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R79bb36df37cf40cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R64ca086bbac04020"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,8 +404,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N25"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N26"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R310f084cce9c4403"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R579b75c367084532"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2513,47 +2513,91 @@
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
-      <x:c r="A25" s="39" t="str">
+      <x:c r="A25" s="35" t="str">
         <x:v>US-039</x:v>
       </x:c>
-      <x:c r="B25" s="40" t="str">
-        <x:v>Story</x:v>
-      </x:c>
-      <x:c r="C25" s="40" t="str">
+      <x:c r="B25" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C25" s="36" t="str">
         <x:v>Future MIDI En DAW Integratie</x:v>
       </x:c>
-      <x:c r="D25" s="40" t="str">
+      <x:c r="D25" s="36" t="str">
         <x:v>Sustain Pedal CC64</x:v>
       </x:c>
-      <x:c r="E25" s="40" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="F25" s="40" t="str">
-        <x:v>Must</x:v>
-      </x:c>
-      <x:c r="G25" s="40" t="str">
+      <x:c r="E25" s="36" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F25" s="36" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="G25" s="36" t="str">
         <x:v>DSP Engineer</x:v>
       </x:c>
-      <x:c r="H25" s="41" t="n">
+      <x:c r="H25" s="37" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="I25" s="40" t="str">
+      <x:c r="I25" s="36" t="str">
         <x:v>Future</x:v>
       </x:c>
-      <x:c r="J25" s="40" t="str">
+      <x:c r="J25" s="36" t="str">
         <x:v>CC64 sustain pedal houdt released sustained voices vast tot pedal up.</x:v>
       </x:c>
-      <x:c r="K25" s="40" t="str">
+      <x:c r="K25" s="36" t="str">
         <x:v>CC64 down/up, held note release, CLI diagnostics en docs tests falen.</x:v>
       </x:c>
-      <x:c r="L25" s="40" t="str">
+      <x:c r="L25" s="36" t="str">
         <x:v>control_change:64 handling in sustained mode, pedal threshold 64 en docs/sustain_pedal_cc64_v0.1.0.md.</x:v>
       </x:c>
-      <x:c r="M25" s="40" t="str">
+      <x:c r="M25" s="36" t="str">
         <x:v>US-035, US-038</x:v>
       </x:c>
-      <x:c r="N25" s="42" t="str">
+      <x:c r="N25" s="38" t="str">
         <x:v>PO accepteerde zonder fysieke sustain pedal, op basis van aanname plus groene automatische CC64-tests.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="39" t="str">
+        <x:v>US-040</x:v>
+      </x:c>
+      <x:c r="B26" s="40" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C26" s="40" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D26" s="40" t="str">
+        <x:v>Envelope Release / Soft Note-Off</x:v>
+      </x:c>
+      <x:c r="E26" s="40" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="F26" s="40" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="G26" s="40" t="str">
+        <x:v>DSP Engineer</x:v>
+      </x:c>
+      <x:c r="H26" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I26" s="40" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J26" s="40" t="str">
+        <x:v>note-off en sustain pedal release stoppen met korte fade-out in plaats van hard afkappen.</x:v>
+      </x:c>
+      <x:c r="K26" s="40" t="str">
+        <x:v>release-time, sustained audio envelope, CLI diagnostics en docs tests falen.</x:v>
+      </x:c>
+      <x:c r="L26" s="40" t="str">
+        <x:v>SustainedVoiceState release frames, --release-time en soft note-off docs/tests.</x:v>
+      </x:c>
+      <x:c r="M26" s="40" t="str">
+        <x:v>US-035, US-039</x:v>
+      </x:c>
+      <x:c r="N26" s="42" t="str">
+        <x:v>In review: default release_time=0.03s; --release-time 0 zet hard stop terug.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2574,7 +2618,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49bcad945a6045b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2beec844e1744e59"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2722,8 +2766,8 @@
         <x:v>Future MIDI/DAW Stories</x:v>
       </x:c>
       <x:c r="B9" s="44" t="n">
-        <x:f>COUNTA('Future MIDI DAW'!A5:A25)</x:f>
-        <x:v>21</x:v>
+        <x:f>COUNTA('Future MIDI DAW'!A5:A26)</x:f>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2731,8 +2775,8 @@
         <x:v>Future MIDI/DAW Points</x:v>
       </x:c>
       <x:c r="B10" s="44" t="n">
-        <x:f>SUM('Future MIDI DAW'!H5:H25)</x:f>
-        <x:v>112</x:v>
+        <x:f>SUM('Future MIDI DAW'!H5:H26)</x:f>
+        <x:v>117</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
Add US-041 ADSR envelope parameters
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Re9d971983a9747b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R96764cc598974354"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Re269bd9868af41ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R3d487d922e8c46ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R3d10e323102c4936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rfa0cef43f7ed4b4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rb40193f7c12c42ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R7c421f3e6b9841ac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,8 +404,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N26"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N27"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82b86ed8d8694eb3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc2f2d8fd9c94ec7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2557,47 +2557,91 @@
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
-      <x:c r="A26" s="39" t="str">
+      <x:c r="A26" s="35" t="str">
         <x:v>US-040</x:v>
       </x:c>
-      <x:c r="B26" s="40" t="str">
-        <x:v>Story</x:v>
-      </x:c>
-      <x:c r="C26" s="40" t="str">
+      <x:c r="B26" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C26" s="36" t="str">
         <x:v>Future MIDI En DAW Integratie</x:v>
       </x:c>
-      <x:c r="D26" s="40" t="str">
+      <x:c r="D26" s="36" t="str">
         <x:v>Envelope Release / Soft Note-Off</x:v>
       </x:c>
-      <x:c r="E26" s="40" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="F26" s="40" t="str">
+      <x:c r="E26" s="36" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F26" s="36" t="str">
         <x:v>Should</x:v>
       </x:c>
-      <x:c r="G26" s="40" t="str">
+      <x:c r="G26" s="36" t="str">
         <x:v>DSP Engineer</x:v>
       </x:c>
-      <x:c r="H26" s="41" t="n">
+      <x:c r="H26" s="37" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="I26" s="40" t="str">
+      <x:c r="I26" s="36" t="str">
         <x:v>Future</x:v>
       </x:c>
-      <x:c r="J26" s="40" t="str">
+      <x:c r="J26" s="36" t="str">
         <x:v>note-off en sustain pedal release stoppen met korte fade-out in plaats van hard afkappen.</x:v>
       </x:c>
-      <x:c r="K26" s="40" t="str">
+      <x:c r="K26" s="36" t="str">
         <x:v>release-time, sustained audio envelope, CLI diagnostics en docs tests falen.</x:v>
       </x:c>
-      <x:c r="L26" s="40" t="str">
+      <x:c r="L26" s="36" t="str">
         <x:v>SustainedVoiceState release frames, --release-time en soft note-off docs/tests.</x:v>
       </x:c>
-      <x:c r="M26" s="40" t="str">
+      <x:c r="M26" s="36" t="str">
         <x:v>US-035, US-039</x:v>
       </x:c>
-      <x:c r="N26" s="42" t="str">
+      <x:c r="N26" s="38" t="str">
         <x:v>PO accepteerde US-040 op 2026-07-12; default release_time=0.03s en --release-time 0 zet hard stop terug.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="39" t="str">
+        <x:v>US-041</x:v>
+      </x:c>
+      <x:c r="B27" s="40" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C27" s="40" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D27" s="40" t="str">
+        <x:v>Amp Envelope ADSR Parameters</x:v>
+      </x:c>
+      <x:c r="E27" s="40" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="F27" s="40" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="G27" s="40" t="str">
+        <x:v>DSP Engineer</x:v>
+      </x:c>
+      <x:c r="H27" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I27" s="40" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J27" s="40" t="str">
+        <x:v>Attack, decay, sustain en release vormen de amplitude van sustained voices.</x:v>
+      </x:c>
+      <x:c r="K27" s="40" t="str">
+        <x:v>ADSR settings validation, audio callback envelope, CLI diagnostics en docs tests falen.</x:v>
+      </x:c>
+      <x:c r="L27" s="40" t="str">
+        <x:v>SustainedAudioPlayerSettings ADSR velden, --attack-time, --decay-time, --sustain-level en docs/amp_envelope_adsr_parameters_v0.1.0.md.</x:v>
+      </x:c>
+      <x:c r="M27" s="40" t="str">
+        <x:v>US-040</x:v>
+      </x:c>
+      <x:c r="N27" s="42" t="str">
+        <x:v>In review: commandline ADSR parameters, geen filter envelope, GUI of plugin scope.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2618,7 +2662,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a4a34ffc3fc4fbd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36c35c36b5604d76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2766,8 +2810,8 @@
         <x:v>Future MIDI/DAW Stories</x:v>
       </x:c>
       <x:c r="B9" s="44" t="n">
-        <x:f>COUNTA('Future MIDI DAW'!A5:A26)</x:f>
-        <x:v>22</x:v>
+        <x:f>COUNTA('Future MIDI DAW'!A5:A27)</x:f>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2775,8 +2819,8 @@
         <x:v>Future MIDI/DAW Points</x:v>
       </x:c>
       <x:c r="B10" s="44" t="n">
-        <x:f>SUM('Future MIDI DAW'!H5:H26)</x:f>
-        <x:v>117</x:v>
+        <x:f>SUM('Future MIDI DAW'!H5:H27)</x:f>
+        <x:v>122</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
Add US-042 MIDI performance YAML config
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Red510f0dd3c14d56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rfb0cb2bbb6ae4549"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R6b145f737f0c4de9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R15302c8fa2db4633"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="Rbad63ed63f774181"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rddda0a63db98423c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R94744d6563984bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R546cd697f0e14624"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,8 +404,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:N27"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FutureMidiDawBacklog" displayName="FutureMidiDawBacklog" ref="A4:N28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:N28"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Type"/>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reeba90edda4841d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd12d59ecaeda4169"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2601,47 +2601,91 @@
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
-      <x:c r="A27" s="39" t="str">
+      <x:c r="A27" s="35" t="str">
         <x:v>US-041</x:v>
       </x:c>
-      <x:c r="B27" s="40" t="str">
-        <x:v>Story</x:v>
-      </x:c>
-      <x:c r="C27" s="40" t="str">
+      <x:c r="B27" s="36" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C27" s="36" t="str">
         <x:v>Future MIDI En DAW Integratie</x:v>
       </x:c>
-      <x:c r="D27" s="40" t="str">
+      <x:c r="D27" s="36" t="str">
         <x:v>Amp Envelope ADSR Parameters</x:v>
       </x:c>
-      <x:c r="E27" s="40" t="str">
-        <x:v>Done</x:v>
-      </x:c>
-      <x:c r="F27" s="40" t="str">
+      <x:c r="E27" s="36" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F27" s="36" t="str">
         <x:v>Should</x:v>
       </x:c>
-      <x:c r="G27" s="40" t="str">
+      <x:c r="G27" s="36" t="str">
         <x:v>DSP Engineer</x:v>
       </x:c>
-      <x:c r="H27" s="41" t="n">
+      <x:c r="H27" s="37" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="I27" s="40" t="str">
+      <x:c r="I27" s="36" t="str">
         <x:v>Future</x:v>
       </x:c>
-      <x:c r="J27" s="40" t="str">
+      <x:c r="J27" s="36" t="str">
         <x:v>Attack, decay, sustain en release vormen de amplitude van sustained voices.</x:v>
       </x:c>
-      <x:c r="K27" s="40" t="str">
+      <x:c r="K27" s="36" t="str">
         <x:v>ADSR settings validation, audio callback envelope, CLI diagnostics en docs tests falen.</x:v>
       </x:c>
-      <x:c r="L27" s="40" t="str">
+      <x:c r="L27" s="36" t="str">
         <x:v>SustainedAudioPlayerSettings ADSR velden, --attack-time, --decay-time, --sustain-level en docs/amp_envelope_adsr_parameters_v0.1.0.md.</x:v>
       </x:c>
-      <x:c r="M27" s="40" t="str">
+      <x:c r="M27" s="36" t="str">
         <x:v>US-040</x:v>
       </x:c>
-      <x:c r="N27" s="42" t="str">
+      <x:c r="N27" s="38" t="str">
         <x:v>PO accepteerde US-041 op 2026-07-13; commandline ADSR parameters, geen filter envelope, GUI of plugin scope.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="39" t="str">
+        <x:v>US-042</x:v>
+      </x:c>
+      <x:c r="B28" s="40" t="str">
+        <x:v>Story</x:v>
+      </x:c>
+      <x:c r="C28" s="40" t="str">
+        <x:v>Future MIDI En DAW Integratie</x:v>
+      </x:c>
+      <x:c r="D28" s="40" t="str">
+        <x:v>MIDI Performance Patch YAML Config</x:v>
+      </x:c>
+      <x:c r="E28" s="40" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="F28" s="40" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="G28" s="40" t="str">
+        <x:v>Lead Developer</x:v>
+      </x:c>
+      <x:c r="H28" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I28" s="40" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="J28" s="40" t="str">
+        <x:v>midi play-stream kan performance parameters uit YAML laden met CLI override.</x:v>
+      </x:c>
+      <x:c r="K28" s="40" t="str">
+        <x:v>Config loader, CLI precedence, docs tests en Kanban tests falen.</x:v>
+      </x:c>
+      <x:c r="L28" s="40" t="str">
+        <x:v>MidiPerformanceConfig, play-stream --config, examples/midi_performance_patch.yaml en docs.</x:v>
+      </x:c>
+      <x:c r="M28" s="40" t="str">
+        <x:v>US-041</x:v>
+      </x:c>
+      <x:c r="N28" s="42" t="str">
+        <x:v>In review: YAML defaults voor live performance, CLI flags blijven winnen en device names blijven runtime keuzes.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2662,7 +2706,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7ab2f3adf6a4cf0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d59950ead4241d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2810,8 +2854,8 @@
         <x:v>Future MIDI/DAW Stories</x:v>
       </x:c>
       <x:c r="B9" s="44" t="n">
-        <x:f>COUNTA('Future MIDI DAW'!A5:A27)</x:f>
-        <x:v>23</x:v>
+        <x:f>COUNTA('Future MIDI DAW'!A5:A28)</x:f>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2819,8 +2863,8 @@
         <x:v>Future MIDI/DAW Points</x:v>
       </x:c>
       <x:c r="B10" s="44" t="n">
-        <x:f>SUM('Future MIDI DAW'!H5:H27)</x:f>
-        <x:v>122</x:v>
+        <x:f>SUM('Future MIDI DAW'!H5:H28)</x:f>
+        <x:v>127</x:v>
       </x:c>
     </x:row>
     <x:row r="11">

</xml_diff>

<commit_message>
Add MVP review pack
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
+++ b/outputs/CHATOD-20260709-D1PY-MVP-001/python_d1_synth_sprint_1_kanban_backlog.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R1188c21d21f54000"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="Rb15a12d0c80849bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R59173c9813f74742"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="R9d5b3a64294b4a8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1 Board" sheetId="1" r:id="R258104c3b4c445f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future MIDI DAW" sheetId="2" r:id="R20626753b9634015"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rc4ba64ab1a3344ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" r:id="Rb2ad13f0cac64ef0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -657,7 +657,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="5" t="str">
-        <x:v>ChatOD: CHATOD-20260709-D1PY-MVP-001 | Date: 2026-07-09 | Status: Draft for customer review</x:v>
+        <x:v>ChatOD: CHATOD-20260709-D1PY-MVP-001 | MVP accepted: 2026-07-14 | Stories: US-001 through US-042</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -1527,7 +1527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb15488ce35464e5b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62897b8a49b54900"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1572,7 +1572,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="28" t="str">
-        <x:v>Scope mutation: Logic Pro 12.3, other DAWs, generic USB MIDI, external MIDI, RaspiMidiHub, physical MIDI hub, MiniFreak, Arturia KeyLab Mk3, Fishman TriplePlay, M-Vave</x:v>
+        <x:v>MVP accepted on 2026-07-14: Logic Pro External MIDI to python-d1-synth with YAML-driven performance config. Future options: synth character, usability, delivery, plugin feasibility, hardware feasibility.</x:v>
       </x:c>
       <x:c r="B2" s="28"/>
       <x:c r="C2" s="28"/>
@@ -2706,7 +2706,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d951cd285214ccd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2e1efea2e9244a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>